<commit_message>
add changes to Excel sheets
</commit_message>
<xml_diff>
--- a/Calibrations/LoadCalibration_2026-01-06_162625.xlsx
+++ b/Calibrations/LoadCalibration_2026-01-06_162625.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\milli079\Documents\GitHub\SAFL-Mesocosms\Calibrations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38A16201-9288-4C2D-918C-150499202228}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{585E69B7-B35A-4C5F-AF2D-1CCEE7860F1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{B7532992-699C-4FBA-BAEA-5C2B991C3C2C}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="17385" xr2:uid="{B7532992-699C-4FBA-BAEA-5C2B991C3C2C}"/>
   </bookViews>
   <sheets>
     <sheet name="LoadCalibration_2026-01-06_1626" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -821,7 +821,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
@@ -837,7 +837,6 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2830,7 +2829,7 @@
       <c r="M34" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="N34" s="15" t="s">
+      <c r="N34" s="14" t="s">
         <v>48</v>
       </c>
     </row>
@@ -2843,7 +2842,7 @@
         <f t="shared" ref="C35:C54" si="10">R11*453.59237</f>
         <v>0</v>
       </c>
-      <c r="D35" s="7">
+      <c r="D35" s="3">
         <f>C35-B35</f>
         <v>0</v>
       </c>
@@ -2872,12 +2871,12 @@
         <v>0</v>
       </c>
       <c r="L35" s="3">
-        <f>G11*$N$35+O35</f>
+        <f>G11*$N$35+$O$35</f>
         <v>-10.0193861542501</v>
       </c>
       <c r="M35" s="3">
-        <f>L35-H35</f>
-        <v>-10.0193861542501</v>
+        <f>ABS(L35-H35)</f>
+        <v>10.0193861542501</v>
       </c>
       <c r="N35" cm="1">
         <f t="array" ref="N35:O35">LINEST(H35:H54,G11:G30)</f>
@@ -2896,8 +2895,8 @@
         <f t="shared" si="10"/>
         <v>4076.6612594394715</v>
       </c>
-      <c r="D36" s="5">
-        <f t="shared" ref="D36:D54" si="16">C36-B36</f>
+      <c r="D36" s="3">
+        <f>ABS(C36-B36)</f>
         <v>12.473624239471064</v>
       </c>
       <c r="E36" s="5">
@@ -2909,7 +2908,7 @@
         <v>2722.7992517146326</v>
       </c>
       <c r="G36" s="5">
-        <f t="shared" ref="G36:G54" si="17">F36-E36</f>
+        <f>ABS(F36-E36)</f>
         <v>10.316879114632229</v>
       </c>
       <c r="H36" s="5">
@@ -2921,16 +2920,16 @@
         <v>0</v>
       </c>
       <c r="J36" s="5">
-        <f t="shared" ref="J36:J54" si="18">I36-H36</f>
+        <f>ABS(I36-H36)</f>
         <v>0</v>
       </c>
       <c r="L36" s="3">
-        <f t="shared" ref="L36:L54" si="19">G12*$N$35+O36</f>
-        <v>75.365616618985001</v>
+        <f t="shared" ref="L36:L54" si="16">G12*$N$35+$O$35</f>
+        <v>-10.0193861542501</v>
       </c>
       <c r="M36" s="3">
-        <f t="shared" ref="M36:M54" si="20">L36-H36</f>
-        <v>75.365616618985001</v>
+        <f t="shared" ref="M36:M54" si="17">ABS(L36-H36)</f>
+        <v>10.0193861542501</v>
       </c>
     </row>
     <row r="37" spans="2:15" x14ac:dyDescent="0.25">
@@ -2942,8 +2941,8 @@
         <f t="shared" si="10"/>
         <v>4068.0968450288842</v>
       </c>
-      <c r="D37" s="5">
-        <f t="shared" si="16"/>
+      <c r="D37" s="3">
+        <f t="shared" ref="D37:D54" si="18">ABS(C37-B37)</f>
         <v>3.9092098288838315</v>
       </c>
       <c r="E37" s="5">
@@ -2955,7 +2954,7 @@
         <v>2733.8450904639822</v>
       </c>
       <c r="G37" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" ref="G37:G54" si="19">ABS(F37-E37)</f>
         <v>21.362717863981743</v>
       </c>
       <c r="H37" s="5">
@@ -2967,16 +2966,16 @@
         <v>821.17284553662125</v>
       </c>
       <c r="J37" s="5">
-        <f t="shared" si="18"/>
+        <f t="shared" ref="J37:J54" si="20">ABS(I37-H37)</f>
         <v>18.31435063662127</v>
       </c>
       <c r="L37" s="3">
-        <f t="shared" si="19"/>
-        <v>889.31427610402295</v>
+        <f t="shared" si="16"/>
+        <v>803.92927333078785</v>
       </c>
       <c r="M37" s="3">
-        <f t="shared" si="20"/>
-        <v>86.455781204022969</v>
+        <f t="shared" si="17"/>
+        <v>1.0707784307878683</v>
       </c>
     </row>
     <row r="38" spans="2:15" x14ac:dyDescent="0.25">
@@ -2988,8 +2987,8 @@
         <f t="shared" si="10"/>
         <v>4082.3708690465301</v>
       </c>
-      <c r="D38" s="5">
-        <f t="shared" si="16"/>
+      <c r="D38" s="3">
+        <f t="shared" si="18"/>
         <v>18.183233846529674</v>
       </c>
       <c r="E38" s="5">
@@ -3001,7 +3000,7 @@
         <v>2744.8909292133321</v>
       </c>
       <c r="G38" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>32.408556613331712</v>
       </c>
       <c r="H38" s="5">
@@ -3013,16 +3012,16 @@
         <v>2357.0702047810428</v>
       </c>
       <c r="J38" s="5">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>11.997651881042657</v>
       </c>
       <c r="L38" s="3">
-        <f t="shared" si="19"/>
-        <v>2411.69973180752</v>
+        <f t="shared" si="16"/>
+        <v>2326.3147290342849</v>
       </c>
       <c r="M38" s="3">
-        <f t="shared" si="20"/>
-        <v>66.627178907519919</v>
+        <f t="shared" si="17"/>
+        <v>18.757823865715181</v>
       </c>
     </row>
     <row r="39" spans="2:15" x14ac:dyDescent="0.25">
@@ -3034,8 +3033,8 @@
         <f t="shared" si="10"/>
         <v>4090.9352834571168</v>
       </c>
-      <c r="D39" s="5">
-        <f t="shared" si="16"/>
+      <c r="D39" s="3">
+        <f t="shared" si="18"/>
         <v>26.747648257116452</v>
       </c>
       <c r="E39" s="5">
@@ -3047,7 +3046,7 @@
         <v>2714.5148726526204</v>
       </c>
       <c r="G39" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>2.0325000526199801</v>
       </c>
       <c r="H39" s="5">
@@ -3059,16 +3058,16 @@
         <v>5155.1406414243447</v>
       </c>
       <c r="J39" s="5">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>52.226478924344519</v>
       </c>
       <c r="L39" s="3">
-        <f t="shared" si="19"/>
-        <v>5185.1544233861678</v>
+        <f t="shared" si="16"/>
+        <v>5099.7694206129327</v>
       </c>
       <c r="M39" s="3">
-        <f t="shared" si="20"/>
-        <v>82.240260886167562</v>
+        <f t="shared" si="17"/>
+        <v>3.1447418870675392</v>
       </c>
     </row>
     <row r="40" spans="2:15" x14ac:dyDescent="0.25">
@@ -3080,8 +3079,8 @@
         <f t="shared" si="10"/>
         <v>4082.3708690465301</v>
       </c>
-      <c r="D40" s="5">
-        <f t="shared" si="16"/>
+      <c r="D40" s="3">
+        <f t="shared" si="18"/>
         <v>18.183233846529674</v>
       </c>
       <c r="E40" s="5">
@@ -3093,7 +3092,7 @@
         <v>2722.7992517146326</v>
       </c>
       <c r="G40" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>10.316879114632229</v>
       </c>
       <c r="H40" s="5">
@@ -3105,16 +3104,16 @@
         <v>8683.1424963224217</v>
       </c>
       <c r="J40" s="5">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>83.031161122420599</v>
       </c>
       <c r="L40" s="3">
-        <f t="shared" si="19"/>
-        <v>8682.1190345070718</v>
+        <f t="shared" si="16"/>
+        <v>8596.7340317338367</v>
       </c>
       <c r="M40" s="3">
-        <f t="shared" si="20"/>
-        <v>82.007699307070652</v>
+        <f t="shared" si="17"/>
+        <v>3.3773034661644488</v>
       </c>
     </row>
     <row r="41" spans="2:15" x14ac:dyDescent="0.25">
@@ -3126,8 +3125,8 @@
         <f t="shared" si="10"/>
         <v>4079.5160642430005</v>
       </c>
-      <c r="D41" s="5">
-        <f t="shared" si="16"/>
+      <c r="D41" s="3">
+        <f t="shared" si="18"/>
         <v>15.328429043000142</v>
       </c>
       <c r="E41" s="5">
@@ -3139,7 +3138,7 @@
         <v>2720.0377920272958</v>
       </c>
       <c r="G41" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>7.5554194272954192</v>
       </c>
       <c r="H41" s="5">
@@ -3151,16 +3150,16 @@
         <v>12560.90315580091</v>
       </c>
       <c r="J41" s="5">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>109.7925993009103</v>
       </c>
       <c r="L41" s="3">
-        <f t="shared" si="19"/>
-        <v>12525.765482075307</v>
+        <f t="shared" si="16"/>
+        <v>12440.380479302072</v>
       </c>
       <c r="M41" s="3">
-        <f t="shared" si="20"/>
-        <v>74.654925575307061</v>
+        <f t="shared" si="17"/>
+        <v>10.73007719792804</v>
       </c>
     </row>
     <row r="42" spans="2:15" x14ac:dyDescent="0.25">
@@ -3172,8 +3171,8 @@
         <f t="shared" si="10"/>
         <v>4070.9516498324128</v>
       </c>
-      <c r="D42" s="5">
-        <f t="shared" si="16"/>
+      <c r="D42" s="3">
+        <f t="shared" si="18"/>
         <v>6.7640146324124544</v>
       </c>
       <c r="E42" s="5">
@@ -3185,7 +3184,7 @@
         <v>2733.8450904639822</v>
       </c>
       <c r="G42" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>21.362717863981743</v>
       </c>
       <c r="H42" s="5">
@@ -3197,16 +3196,16 @@
         <v>15936.83596522924</v>
       </c>
       <c r="J42" s="5">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>142.74964182923941</v>
       </c>
       <c r="L42" s="3">
-        <f t="shared" si="19"/>
-        <v>15871.998859958239</v>
+        <f t="shared" si="16"/>
+        <v>15786.613857185004</v>
       </c>
       <c r="M42" s="3">
-        <f t="shared" si="20"/>
-        <v>77.912536558238571</v>
+        <f t="shared" si="17"/>
+        <v>7.4724662149965297</v>
       </c>
     </row>
     <row r="43" spans="2:15" x14ac:dyDescent="0.25">
@@ -3218,8 +3217,8 @@
         <f t="shared" si="10"/>
         <v>4082.3708690465301</v>
       </c>
-      <c r="D43" s="5">
-        <f t="shared" si="16"/>
+      <c r="D43" s="3">
+        <f t="shared" si="18"/>
         <v>18.183233846529674</v>
       </c>
       <c r="E43" s="5">
@@ -3231,7 +3230,7 @@
         <v>2717.2763323399581</v>
       </c>
       <c r="G43" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>4.7939597399576996</v>
       </c>
       <c r="H43" s="5">
@@ -3243,16 +3242,16 @@
         <v>18309.113074557259</v>
       </c>
       <c r="J43" s="5">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>174.49012195726027</v>
       </c>
       <c r="L43" s="3">
-        <f t="shared" si="19"/>
-        <v>18223.406098470572</v>
+        <f t="shared" si="16"/>
+        <v>18138.021095697339</v>
       </c>
       <c r="M43" s="3">
-        <f t="shared" si="20"/>
-        <v>88.783145870573208</v>
+        <f t="shared" si="17"/>
+        <v>3.3981430973399256</v>
       </c>
     </row>
     <row r="44" spans="2:15" x14ac:dyDescent="0.25">
@@ -3264,8 +3263,8 @@
         <f t="shared" si="10"/>
         <v>4076.6612594394715</v>
       </c>
-      <c r="D44" s="5">
-        <f t="shared" si="16"/>
+      <c r="D44" s="3">
+        <f t="shared" si="18"/>
         <v>12.473624239471064</v>
       </c>
       <c r="E44" s="5">
@@ -3277,8 +3276,8 @@
         <v>2711.7534129652836</v>
       </c>
       <c r="G44" s="5">
-        <f t="shared" si="17"/>
-        <v>-0.7289596347168299</v>
+        <f t="shared" si="19"/>
+        <v>0.7289596347168299</v>
       </c>
       <c r="H44" s="5">
         <f t="shared" si="13"/>
@@ -3289,16 +3288,16 @@
         <v>20574.941852056458</v>
       </c>
       <c r="J44" s="5">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>176.89297315645672</v>
       </c>
       <c r="L44" s="3">
-        <f t="shared" si="19"/>
-        <v>20469.301473716325</v>
+        <f t="shared" si="16"/>
+        <v>20383.916470943092</v>
       </c>
       <c r="M44" s="3">
-        <f t="shared" si="20"/>
-        <v>71.252594816323835</v>
+        <f t="shared" si="17"/>
+        <v>14.132407956909447</v>
       </c>
     </row>
     <row r="45" spans="2:15" x14ac:dyDescent="0.25">
@@ -3310,8 +3309,8 @@
         <f t="shared" si="10"/>
         <v>4093.7900882606455</v>
       </c>
-      <c r="D45" s="5">
-        <f t="shared" si="16"/>
+      <c r="D45" s="3">
+        <f t="shared" si="18"/>
         <v>29.602453060645075</v>
       </c>
       <c r="E45" s="5">
@@ -3323,7 +3322,7 @@
         <v>2722.7992517146326</v>
       </c>
       <c r="G45" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>10.316879114632229</v>
       </c>
       <c r="H45" s="5">
@@ -3335,16 +3334,16 @@
         <v>22019.597784019032</v>
       </c>
       <c r="J45" s="5">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>215.41255811903102</v>
       </c>
       <c r="L45" s="3">
-        <f t="shared" si="19"/>
-        <v>21901.248189477039</v>
+        <f t="shared" si="16"/>
+        <v>21815.863186703806</v>
       </c>
       <c r="M45" s="3">
-        <f t="shared" si="20"/>
-        <v>97.062963577038317</v>
+        <f t="shared" si="17"/>
+        <v>11.677960803805036</v>
       </c>
     </row>
     <row r="46" spans="2:15" x14ac:dyDescent="0.25">
@@ -3356,8 +3355,8 @@
         <f t="shared" si="10"/>
         <v>4088.0804786535878</v>
       </c>
-      <c r="D46" s="5">
-        <f t="shared" si="16"/>
+      <c r="D46" s="3">
+        <f t="shared" si="18"/>
         <v>23.892843453587375</v>
       </c>
       <c r="E46" s="5">
@@ -3369,7 +3368,7 @@
         <v>0</v>
       </c>
       <c r="G46" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="H46" s="5">
@@ -3381,16 +3380,16 @@
         <v>22019.597784019032</v>
       </c>
       <c r="J46" s="5">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>215.41255811903102</v>
       </c>
       <c r="L46" s="3">
-        <f t="shared" si="19"/>
-        <v>21901.248189477039</v>
+        <f t="shared" si="16"/>
+        <v>21815.863186703806</v>
       </c>
       <c r="M46" s="3">
-        <f t="shared" si="20"/>
-        <v>97.062963577038317</v>
+        <f t="shared" si="17"/>
+        <v>11.677960803805036</v>
       </c>
     </row>
     <row r="47" spans="2:15" x14ac:dyDescent="0.25">
@@ -3402,8 +3401,8 @@
         <f t="shared" si="10"/>
         <v>4096.6448930641745</v>
       </c>
-      <c r="D47" s="5">
-        <f t="shared" si="16"/>
+      <c r="D47" s="3">
+        <f t="shared" si="18"/>
         <v>32.457257864174153</v>
       </c>
       <c r="E47" s="5">
@@ -3415,7 +3414,7 @@
         <v>2722.7992517146326</v>
       </c>
       <c r="G47" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>10.316879114632229</v>
       </c>
       <c r="H47" s="5">
@@ -3427,16 +3426,16 @@
         <v>16545.112147108222</v>
       </c>
       <c r="J47" s="5">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>143.2120479082223</v>
       </c>
       <c r="L47" s="3">
-        <f t="shared" si="19"/>
-        <v>16474.923792910118</v>
+        <f t="shared" si="16"/>
+        <v>16389.538790136881</v>
       </c>
       <c r="M47" s="3">
-        <f t="shared" si="20"/>
-        <v>73.023693710118096</v>
+        <f t="shared" si="17"/>
+        <v>12.361309063118824</v>
       </c>
     </row>
     <row r="48" spans="2:15" x14ac:dyDescent="0.25">
@@ -3448,8 +3447,8 @@
         <f t="shared" si="10"/>
         <v>4068.0968450288842</v>
       </c>
-      <c r="D48" s="5">
-        <f t="shared" si="16"/>
+      <c r="D48" s="3">
+        <f t="shared" si="18"/>
         <v>3.9092098288838315</v>
       </c>
       <c r="E48" s="5">
@@ -3461,7 +3460,7 @@
         <v>2722.7992517146326</v>
       </c>
       <c r="G48" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>10.316879114632229</v>
       </c>
       <c r="H48" s="5">
@@ -3473,16 +3472,16 @@
         <v>12591.316964894861</v>
       </c>
       <c r="J48" s="5">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>117.52678989486049</v>
       </c>
       <c r="L48" s="3">
-        <f t="shared" si="19"/>
-        <v>12555.9117287229</v>
+        <f t="shared" si="16"/>
+        <v>12470.526725949665</v>
       </c>
       <c r="M48" s="3">
-        <f t="shared" si="20"/>
-        <v>82.121553722899989</v>
+        <f t="shared" si="17"/>
+        <v>3.2634490503351117</v>
       </c>
     </row>
     <row r="49" spans="2:13" x14ac:dyDescent="0.25">
@@ -3494,8 +3493,8 @@
         <f t="shared" si="10"/>
         <v>4085.2256738500591</v>
       </c>
-      <c r="D49" s="5">
-        <f t="shared" si="16"/>
+      <c r="D49" s="3">
+        <f t="shared" si="18"/>
         <v>21.038038650058752</v>
       </c>
       <c r="E49" s="5">
@@ -3507,7 +3506,7 @@
         <v>2722.7992517146326</v>
       </c>
       <c r="G49" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>10.316879114632229</v>
       </c>
       <c r="H49" s="5">
@@ -3519,16 +3518,16 @@
         <v>8561.4872599466271</v>
       </c>
       <c r="J49" s="5">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>115.59733054662684</v>
       </c>
       <c r="L49" s="3">
-        <f t="shared" si="19"/>
-        <v>8561.5340479166953</v>
+        <f t="shared" si="16"/>
+        <v>8476.1490451434602</v>
       </c>
       <c r="M49" s="3">
-        <f t="shared" si="20"/>
-        <v>115.64411851669502</v>
+        <f t="shared" si="17"/>
+        <v>30.259115743459915</v>
       </c>
     </row>
     <row r="50" spans="2:13" x14ac:dyDescent="0.25">
@@ -3540,8 +3539,8 @@
         <f t="shared" si="10"/>
         <v>4088.0804786535878</v>
       </c>
-      <c r="D50" s="5">
-        <f t="shared" si="16"/>
+      <c r="D50" s="3">
+        <f t="shared" si="18"/>
         <v>23.892843453587375</v>
       </c>
       <c r="E50" s="5">
@@ -3553,7 +3552,7 @@
         <v>2717.2763323399581</v>
       </c>
       <c r="G50" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>4.7939597399576996</v>
       </c>
       <c r="H50" s="5">
@@ -3565,16 +3564,16 @@
         <v>4987.8646914076262</v>
       </c>
       <c r="J50" s="5">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>57.315629507625999</v>
       </c>
       <c r="L50" s="3">
-        <f t="shared" si="19"/>
-        <v>5019.3500668244005</v>
+        <f t="shared" si="16"/>
+        <v>4933.9650640511654</v>
       </c>
       <c r="M50" s="3">
-        <f t="shared" si="20"/>
-        <v>88.801004924400331</v>
+        <f t="shared" si="17"/>
+        <v>3.4160021511652303</v>
       </c>
     </row>
     <row r="51" spans="2:13" x14ac:dyDescent="0.25">
@@ -3586,8 +3585,8 @@
         <f t="shared" si="10"/>
         <v>4085.2256738500591</v>
       </c>
-      <c r="D51" s="5">
-        <f t="shared" si="16"/>
+      <c r="D51" s="3">
+        <f t="shared" si="18"/>
         <v>21.038038650058752</v>
       </c>
       <c r="E51" s="5">
@@ -3599,7 +3598,7 @@
         <v>2722.7992517146326</v>
       </c>
       <c r="G51" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>10.316879114632229</v>
       </c>
       <c r="H51" s="5">
@@ -3611,16 +3610,16 @@
         <v>2326.6563956870941</v>
       </c>
       <c r="J51" s="5">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>36.014927187094145</v>
       </c>
       <c r="L51" s="3">
-        <f t="shared" si="19"/>
-        <v>2381.5534851599259</v>
+        <f t="shared" si="16"/>
+        <v>2296.1684823866908</v>
       </c>
       <c r="M51" s="3">
-        <f t="shared" si="20"/>
-        <v>90.912016659925939</v>
+        <f t="shared" si="17"/>
+        <v>5.5270138866908383</v>
       </c>
     </row>
     <row r="52" spans="2:13" x14ac:dyDescent="0.25">
@@ -3632,8 +3631,8 @@
         <f t="shared" si="10"/>
         <v>4068.0968450288842</v>
       </c>
-      <c r="D52" s="5">
-        <f t="shared" si="16"/>
+      <c r="D52" s="3">
+        <f t="shared" si="18"/>
         <v>3.9092098288838315</v>
       </c>
       <c r="E52" s="5">
@@ -3645,8 +3644,8 @@
         <v>2708.9919532779459</v>
       </c>
       <c r="G52" s="5">
-        <f t="shared" si="17"/>
-        <v>-3.4904193220545494</v>
+        <f t="shared" si="19"/>
+        <v>3.4904193220545494</v>
       </c>
       <c r="H52" s="5">
         <f t="shared" si="13"/>
@@ -3657,16 +3656,16 @@
         <v>836.3797500835957</v>
       </c>
       <c r="J52" s="5">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>33.521255183595713</v>
       </c>
       <c r="L52" s="3">
-        <f t="shared" si="19"/>
-        <v>904.3873994278199</v>
+        <f t="shared" si="16"/>
+        <v>819.0023966545848</v>
       </c>
       <c r="M52" s="3">
-        <f t="shared" si="20"/>
-        <v>101.52890452781992</v>
+        <f t="shared" si="17"/>
+        <v>16.143901754584817</v>
       </c>
     </row>
     <row r="53" spans="2:13" x14ac:dyDescent="0.25">
@@ -3678,8 +3677,8 @@
         <f t="shared" si="10"/>
         <v>4085.2256738500591</v>
       </c>
-      <c r="D53" s="5">
-        <f t="shared" si="16"/>
+      <c r="D53" s="3">
+        <f t="shared" si="18"/>
         <v>21.038038650058752</v>
       </c>
       <c r="E53" s="5">
@@ -3691,7 +3690,7 @@
         <v>2714.5148726526204</v>
       </c>
       <c r="G53" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>2.0325000526199801</v>
       </c>
       <c r="H53" s="5">
@@ -3703,16 +3702,16 @@
         <v>15.206904546974464</v>
       </c>
       <c r="J53" s="5">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>15.206904546974464</v>
       </c>
       <c r="L53" s="3">
-        <f t="shared" si="19"/>
-        <v>90.438739942781993</v>
+        <f t="shared" si="16"/>
+        <v>5.053737169546892</v>
       </c>
       <c r="M53" s="3">
-        <f t="shared" si="20"/>
-        <v>90.438739942781993</v>
+        <f t="shared" si="17"/>
+        <v>5.053737169546892</v>
       </c>
     </row>
     <row r="54" spans="2:13" x14ac:dyDescent="0.25">
@@ -3724,8 +3723,8 @@
         <f t="shared" si="10"/>
         <v>2.8548048035290443</v>
       </c>
-      <c r="D54" s="5">
-        <f t="shared" si="16"/>
+      <c r="D54" s="3">
+        <f t="shared" si="18"/>
         <v>2.8548048035290443</v>
       </c>
       <c r="E54" s="5">
@@ -3737,7 +3736,7 @@
         <v>0</v>
       </c>
       <c r="G54" s="5">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="H54" s="5">
@@ -3749,16 +3748,16 @@
         <v>15.206904546974464</v>
       </c>
       <c r="J54" s="5">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>15.206904546974464</v>
       </c>
       <c r="L54" s="3">
-        <f t="shared" si="19"/>
-        <v>90.438739942781993</v>
+        <f t="shared" si="16"/>
+        <v>5.053737169546892</v>
       </c>
       <c r="M54" s="3">
-        <f t="shared" si="20"/>
-        <v>90.438739942781993</v>
+        <f t="shared" si="17"/>
+        <v>5.053737169546892</v>
       </c>
     </row>
     <row r="55" spans="2:13" x14ac:dyDescent="0.25">
@@ -3774,7 +3773,7 @@
       </c>
       <c r="G55" s="3">
         <f>AVERAGE(G39:G54)</f>
-        <v>6.2658095379659073</v>
+        <v>6.7932319075623298</v>
       </c>
       <c r="I55" t="s">
         <v>40</v>
@@ -3788,7 +3787,7 @@
       </c>
       <c r="M55" s="3">
         <f>AVERAGE(M39:M54)</f>
-        <v>87.742866382198798</v>
+        <v>9.1680829635290308</v>
       </c>
     </row>
     <row r="56" spans="2:13" x14ac:dyDescent="0.25">
@@ -3804,7 +3803,7 @@
       </c>
       <c r="G56" s="3">
         <f>MIN(G40:G54)</f>
-        <v>-3.4904193220545494</v>
+        <v>0</v>
       </c>
       <c r="I56" t="s">
         <v>41</v>
@@ -3818,7 +3817,7 @@
       </c>
       <c r="M56" s="3">
         <f>MIN(M40:M54)</f>
-        <v>71.252594816323835</v>
+        <v>3.2634490503351117</v>
       </c>
     </row>
     <row r="57" spans="2:13" x14ac:dyDescent="0.25">
@@ -3848,11 +3847,23 @@
       </c>
       <c r="M57" s="3">
         <f>MAX(M39:M54)</f>
-        <v>115.64411851669502</v>
+        <v>30.259115743459915</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D35:D54 G35:G54 J35:J54">
+  <conditionalFormatting sqref="G35:G54 J35:J54">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D35:D54">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>

<commit_message>
add changes to Excel calibration summaries
</commit_message>
<xml_diff>
--- a/Calibrations/LoadCalibration_2026-01-06_162625.xlsx
+++ b/Calibrations/LoadCalibration_2026-01-06_162625.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\milli079\Documents\GitHub\SAFL-Mesocosms\Calibrations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{585E69B7-B35A-4C5F-AF2D-1CCEE7860F1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9E59C82-0C58-4E7E-95D6-442D04FF1705}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="17385" xr2:uid="{B7532992-699C-4FBA-BAEA-5C2B991C3C2C}"/>
+    <workbookView xWindow="-24120" yWindow="660" windowWidth="24240" windowHeight="13020" xr2:uid="{B7532992-699C-4FBA-BAEA-5C2B991C3C2C}"/>
   </bookViews>
   <sheets>
     <sheet name="LoadCalibration_2026-01-06_1626" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -1212,7 +1212,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D354759F-62D7-4E5C-8857-5158718CF50F}">
-  <dimension ref="A1:T57"/>
+  <dimension ref="A1:U57"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -1220,10 +1220,12 @@
     <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="9.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.5703125" customWidth="1"/>
+    <col min="11" max="11" width="14.140625" customWidth="1"/>
+    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="E1" t="s">
         <v>12</v>
       </c>
@@ -1233,23 +1235,23 @@
       <c r="G1" t="s">
         <v>27</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>14</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>15</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>16</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>17</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="E2">
         <v>3.1949999999999998</v>
       </c>
@@ -1259,23 +1261,23 @@
       <c r="G2">
         <v>2.9990000000000001</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>19</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>15</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>20</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>17</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="D3" t="s">
         <v>21</v>
       </c>
@@ -1288,23 +1290,23 @@
       <c r="G3">
         <v>4.9729999999999999</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>43</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>44</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>45</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>17</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="D4" t="s">
         <v>26</v>
       </c>
@@ -1317,20 +1319,20 @@
       <c r="G4">
         <v>50</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>22</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>23</v>
       </c>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
         <v>24</v>
       </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="D5" t="s">
         <v>28</v>
       </c>
@@ -1347,7 +1349,7 @@
         <v>3.3525485772554924</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -1369,44 +1371,44 @@
       <c r="G9" t="s">
         <v>6</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>7</v>
       </c>
-      <c r="I9" t="s">
+      <c r="J9" t="s">
         <v>4</v>
       </c>
-      <c r="J9" t="s">
+      <c r="K9" t="s">
         <v>5</v>
       </c>
-      <c r="K9" t="s">
+      <c r="L9" t="s">
         <v>6</v>
       </c>
-      <c r="L9" t="s">
+      <c r="M9" t="s">
         <v>7</v>
       </c>
-      <c r="M9" t="s">
+      <c r="N9" t="s">
         <v>8</v>
       </c>
-      <c r="O9" t="s">
+      <c r="P9" t="s">
         <v>29</v>
       </c>
-      <c r="P9" t="s">
+      <c r="Q9" t="s">
         <v>30</v>
       </c>
-      <c r="Q9" t="s">
+      <c r="R9" t="s">
         <v>34</v>
       </c>
-      <c r="R9" s="2" t="s">
+      <c r="S9" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="S9" s="2" t="s">
+      <c r="T9" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="T9" s="2" t="s">
+      <c r="U9" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>9</v>
       </c>
@@ -1425,11 +1427,8 @@
       <c r="G10" t="s">
         <v>10</v>
       </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>10</v>
-      </c>
-      <c r="I10" t="s">
-        <v>11</v>
       </c>
       <c r="J10" t="s">
         <v>11</v>
@@ -1441,10 +1440,10 @@
         <v>11</v>
       </c>
       <c r="M10" t="s">
+        <v>11</v>
+      </c>
+      <c r="N10" t="s">
         <v>9</v>
-      </c>
-      <c r="O10" t="s">
-        <v>10</v>
       </c>
       <c r="P10" t="s">
         <v>10</v>
@@ -1452,8 +1451,8 @@
       <c r="Q10" t="s">
         <v>10</v>
       </c>
-      <c r="R10" s="2" t="s">
-        <v>33</v>
+      <c r="R10" t="s">
+        <v>10</v>
       </c>
       <c r="S10" s="2" t="s">
         <v>33</v>
@@ -1461,8 +1460,11 @@
       <c r="T10" s="2" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U10" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>46028.68509259259</v>
       </c>
@@ -1485,49 +1487,53 @@
         <v>0.05</v>
       </c>
       <c r="H11">
-        <v>0</v>
+        <f>G11*$G$5</f>
+        <v>0.16762742886277462</v>
       </c>
       <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
         <v>33.9</v>
       </c>
-      <c r="J11">
+      <c r="K11">
         <v>6492.2</v>
       </c>
-      <c r="K11">
+      <c r="L11">
         <v>4.5</v>
       </c>
-      <c r="L11">
-        <v>0</v>
-      </c>
       <c r="M11">
+        <v>0</v>
+      </c>
+      <c r="N11">
         <v>-0.45900000000000002</v>
       </c>
-      <c r="O11">
+      <c r="P11">
         <f>E11-E$11</f>
         <v>0</v>
       </c>
-      <c r="P11">
-        <f t="shared" ref="P11:Q11" si="1">F11-F$11</f>
-        <v>0</v>
-      </c>
       <c r="Q11">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R11" s="4">
-        <f>O11*E$5</f>
+        <f>F11-F$11</f>
+        <v>0</v>
+      </c>
+      <c r="R11">
+        <f>G11-G$11</f>
         <v>0</v>
       </c>
       <c r="S11" s="4">
-        <f t="shared" ref="S11:T11" si="2">P11*F$5</f>
+        <f>P11*E$5</f>
         <v>0</v>
       </c>
       <c r="T11" s="4">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+        <f>Q11*F$5</f>
+        <v>0</v>
+      </c>
+      <c r="U11" s="4">
+        <f>R11*G$5</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>46028.685752314814</v>
       </c>
@@ -1550,49 +1556,53 @@
         <v>0.05</v>
       </c>
       <c r="H12">
-        <v>0</v>
+        <f t="shared" ref="H12:H30" si="1">G12*$G$5</f>
+        <v>0.16762742886277462</v>
       </c>
       <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
         <v>61.7</v>
       </c>
-      <c r="J12">
+      <c r="K12">
         <v>38</v>
       </c>
-      <c r="K12">
+      <c r="L12">
         <v>0.2</v>
       </c>
-      <c r="L12">
-        <v>0</v>
-      </c>
       <c r="M12">
+        <v>0</v>
+      </c>
+      <c r="N12">
         <v>37.118000000000002</v>
       </c>
-      <c r="O12">
+      <c r="P12">
         <f>E12-E$11</f>
         <v>14.280000000000001</v>
       </c>
-      <c r="P12">
-        <f t="shared" ref="P12:P30" si="3">F12-F$11</f>
+      <c r="Q12">
+        <f t="shared" ref="Q12:Q30" si="2">F12-F$11</f>
         <v>9.86</v>
       </c>
-      <c r="Q12">
-        <f t="shared" ref="Q12:Q30" si="4">G12-G$11</f>
-        <v>0</v>
-      </c>
-      <c r="R12" s="4">
-        <f t="shared" ref="R12:R30" si="5">O12*E$5</f>
+      <c r="R12">
+        <f t="shared" ref="R12:R30" si="3">G12-G$11</f>
+        <v>0</v>
+      </c>
+      <c r="S12" s="4">
+        <f t="shared" ref="S12:S30" si="4">P12*E$5</f>
         <v>8.9874996341747799</v>
       </c>
-      <c r="S12" s="4">
-        <f t="shared" ref="S12:S30" si="6">P12*F$5</f>
+      <c r="T12" s="4">
+        <f t="shared" ref="T12:T30" si="5">Q12*F$5</f>
         <v>6.0027448250829982</v>
       </c>
-      <c r="T12" s="4">
-        <f>Q12*G$5</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U12" s="4">
+        <f>R12*G$5</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>46028.686435185184</v>
       </c>
@@ -1615,49 +1625,53 @@
         <v>0.59</v>
       </c>
       <c r="H13">
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>1.9780036605807405</v>
       </c>
       <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
         <v>60.3</v>
       </c>
-      <c r="J13">
+      <c r="K13">
         <v>37.200000000000003</v>
       </c>
-      <c r="K13">
+      <c r="L13">
         <v>2.4</v>
       </c>
-      <c r="L13">
-        <v>0</v>
-      </c>
       <c r="M13">
+        <v>0</v>
+      </c>
+      <c r="N13">
         <v>37.953000000000003</v>
       </c>
-      <c r="O13">
-        <f t="shared" ref="O13:O30" si="7">E13-E$11</f>
+      <c r="P13">
+        <f t="shared" ref="P13:P30" si="6">E13-E$11</f>
         <v>14.25</v>
       </c>
-      <c r="P13">
+      <c r="Q13">
+        <f t="shared" si="2"/>
+        <v>9.8999999999999986</v>
+      </c>
+      <c r="R13">
         <f t="shared" si="3"/>
-        <v>9.8999999999999986</v>
-      </c>
-      <c r="Q13">
+        <v>0.53999999999999992</v>
+      </c>
+      <c r="S13" s="4">
         <f t="shared" si="4"/>
-        <v>0.53999999999999992</v>
-      </c>
-      <c r="R13" s="4">
+        <v>8.9686183324223112</v>
+      </c>
+      <c r="T13" s="4">
         <f t="shared" si="5"/>
-        <v>8.9686183324223112</v>
-      </c>
-      <c r="S13" s="4">
-        <f t="shared" si="6"/>
         <v>6.0270967310671075</v>
       </c>
-      <c r="T13" s="4">
-        <f t="shared" ref="T13:T30" si="8">Q13*G$5</f>
+      <c r="U13" s="4">
+        <f t="shared" ref="U13:U30" si="7">R13*G$5</f>
         <v>1.8103762317179657</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>46028.687141203707</v>
       </c>
@@ -1680,49 +1694,53 @@
         <v>1.6</v>
       </c>
       <c r="H14">
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>5.364077723608788</v>
       </c>
       <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14">
         <v>57.9</v>
       </c>
-      <c r="J14">
+      <c r="K14">
         <v>35.6</v>
       </c>
-      <c r="K14">
+      <c r="L14">
         <v>6.3</v>
       </c>
-      <c r="L14">
-        <v>0</v>
-      </c>
       <c r="M14">
+        <v>0</v>
+      </c>
+      <c r="N14">
         <v>39.56</v>
       </c>
-      <c r="O14">
+      <c r="P14">
+        <f t="shared" si="6"/>
+        <v>14.3</v>
+      </c>
+      <c r="Q14">
+        <f t="shared" si="2"/>
+        <v>9.9400000000000013</v>
+      </c>
+      <c r="R14">
+        <f t="shared" si="3"/>
+        <v>1.55</v>
+      </c>
+      <c r="S14" s="4">
+        <f t="shared" si="4"/>
+        <v>9.0000871686764263</v>
+      </c>
+      <c r="T14" s="4">
+        <f t="shared" si="5"/>
+        <v>6.0514486370512186</v>
+      </c>
+      <c r="U14" s="4">
         <f t="shared" si="7"/>
-        <v>14.3</v>
-      </c>
-      <c r="P14">
-        <f t="shared" si="3"/>
-        <v>9.9400000000000013</v>
-      </c>
-      <c r="Q14">
-        <f t="shared" si="4"/>
-        <v>1.55</v>
-      </c>
-      <c r="R14" s="4">
-        <f t="shared" si="5"/>
-        <v>9.0000871686764263</v>
-      </c>
-      <c r="S14" s="4">
-        <f t="shared" si="6"/>
-        <v>6.0514486370512186</v>
-      </c>
-      <c r="T14" s="4">
-        <f t="shared" si="8"/>
         <v>5.1964502947460129</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>46028.688194444447</v>
       </c>
@@ -1745,49 +1763,53 @@
         <v>3.44</v>
       </c>
       <c r="H15">
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>11.532767105758893</v>
       </c>
       <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15">
         <v>54</v>
       </c>
-      <c r="J15">
+      <c r="K15">
         <v>33.200000000000003</v>
       </c>
-      <c r="K15">
+      <c r="L15">
         <v>12.6</v>
       </c>
-      <c r="L15">
-        <v>0</v>
-      </c>
       <c r="M15">
+        <v>0</v>
+      </c>
+      <c r="N15">
         <v>42.399000000000001</v>
       </c>
-      <c r="O15">
-        <f t="shared" si="7"/>
+      <c r="P15">
+        <f t="shared" si="6"/>
         <v>14.33</v>
       </c>
-      <c r="P15">
+      <c r="Q15">
+        <f t="shared" si="2"/>
+        <v>9.8299999999999983</v>
+      </c>
+      <c r="R15">
         <f t="shared" si="3"/>
-        <v>9.8299999999999983</v>
-      </c>
-      <c r="Q15">
+        <v>3.39</v>
+      </c>
+      <c r="S15" s="4">
         <f t="shared" si="4"/>
-        <v>3.39</v>
-      </c>
-      <c r="R15" s="4">
+        <v>9.0189684704288933</v>
+      </c>
+      <c r="T15" s="4">
         <f t="shared" si="5"/>
-        <v>9.0189684704288933</v>
-      </c>
-      <c r="S15" s="4">
-        <f t="shared" si="6"/>
         <v>5.9844808955949151</v>
       </c>
-      <c r="T15" s="4">
-        <f>Q15*G$5</f>
+      <c r="U15" s="4">
+        <f>R15*G$5</f>
         <v>11.365139676896119</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>46028.688888888886</v>
       </c>
@@ -1810,49 +1832,53 @@
         <v>5.76</v>
       </c>
       <c r="H16">
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>19.310679804991636</v>
       </c>
       <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16">
         <v>49.8</v>
       </c>
-      <c r="J16">
+      <c r="K16">
         <v>30.6</v>
       </c>
-      <c r="K16">
+      <c r="L16">
         <v>19.5</v>
       </c>
-      <c r="L16">
-        <v>0</v>
-      </c>
       <c r="M16">
+        <v>0</v>
+      </c>
+      <c r="N16">
         <v>46.014000000000003</v>
       </c>
-      <c r="O16">
+      <c r="P16">
+        <f t="shared" si="6"/>
+        <v>14.3</v>
+      </c>
+      <c r="Q16">
+        <f t="shared" si="2"/>
+        <v>9.86</v>
+      </c>
+      <c r="R16">
+        <f t="shared" si="3"/>
+        <v>5.71</v>
+      </c>
+      <c r="S16" s="4">
+        <f t="shared" si="4"/>
+        <v>9.0000871686764263</v>
+      </c>
+      <c r="T16" s="4">
+        <f t="shared" si="5"/>
+        <v>6.0027448250829982</v>
+      </c>
+      <c r="U16" s="4">
         <f t="shared" si="7"/>
-        <v>14.3</v>
-      </c>
-      <c r="P16">
-        <f t="shared" si="3"/>
-        <v>9.86</v>
-      </c>
-      <c r="Q16">
-        <f t="shared" si="4"/>
-        <v>5.71</v>
-      </c>
-      <c r="R16" s="4">
-        <f t="shared" si="5"/>
-        <v>9.0000871686764263</v>
-      </c>
-      <c r="S16" s="4">
-        <f t="shared" si="6"/>
-        <v>6.0027448250829982</v>
-      </c>
-      <c r="T16" s="4">
-        <f t="shared" si="8"/>
         <v>19.14305237612886</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>46028.689583333333</v>
       </c>
@@ -1875,49 +1901,53 @@
         <v>8.31</v>
       </c>
       <c r="H17">
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>27.859678676993145</v>
       </c>
       <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17">
         <v>45.8</v>
       </c>
-      <c r="J17">
+      <c r="K17">
         <v>28.2</v>
       </c>
-      <c r="K17">
+      <c r="L17">
         <v>25.8</v>
       </c>
-      <c r="L17">
-        <v>0</v>
-      </c>
       <c r="M17">
+        <v>0</v>
+      </c>
+      <c r="N17">
         <v>49.985999999999997</v>
       </c>
-      <c r="O17">
+      <c r="P17">
+        <f t="shared" si="6"/>
+        <v>14.290000000000001</v>
+      </c>
+      <c r="Q17">
+        <f t="shared" si="2"/>
+        <v>9.8500000000000014</v>
+      </c>
+      <c r="R17">
+        <f t="shared" si="3"/>
+        <v>8.26</v>
+      </c>
+      <c r="S17" s="4">
+        <f t="shared" si="4"/>
+        <v>8.9937934014256022</v>
+      </c>
+      <c r="T17" s="4">
+        <f t="shared" si="5"/>
+        <v>5.996656848586972</v>
+      </c>
+      <c r="U17" s="4">
         <f t="shared" si="7"/>
-        <v>14.290000000000001</v>
-      </c>
-      <c r="P17">
-        <f t="shared" si="3"/>
-        <v>9.8500000000000014</v>
-      </c>
-      <c r="Q17">
-        <f t="shared" si="4"/>
-        <v>8.26</v>
-      </c>
-      <c r="R17" s="4">
-        <f t="shared" si="5"/>
-        <v>8.9937934014256022</v>
-      </c>
-      <c r="S17" s="4">
-        <f t="shared" si="6"/>
-        <v>5.996656848586972</v>
-      </c>
-      <c r="T17" s="4">
-        <f t="shared" si="8"/>
         <v>27.692051248130365</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>46028.690972222219</v>
       </c>
@@ -1940,49 +1970,53 @@
         <v>10.53</v>
       </c>
       <c r="H18">
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>35.302336518500333</v>
       </c>
       <c r="I18">
+        <v>0</v>
+      </c>
+      <c r="J18">
         <v>42.8</v>
       </c>
-      <c r="J18">
+      <c r="K18">
         <v>26.4</v>
       </c>
-      <c r="K18">
+      <c r="L18">
         <v>30.6</v>
       </c>
-      <c r="L18">
-        <v>0</v>
-      </c>
       <c r="M18">
+        <v>0</v>
+      </c>
+      <c r="N18">
         <v>53.442999999999998</v>
       </c>
-      <c r="O18">
+      <c r="P18">
+        <f t="shared" si="6"/>
+        <v>14.26</v>
+      </c>
+      <c r="Q18">
+        <f t="shared" si="2"/>
+        <v>9.8999999999999986</v>
+      </c>
+      <c r="R18">
+        <f t="shared" si="3"/>
+        <v>10.479999999999999</v>
+      </c>
+      <c r="S18" s="4">
+        <f t="shared" si="4"/>
+        <v>8.9749120996731335</v>
+      </c>
+      <c r="T18" s="4">
+        <f t="shared" si="5"/>
+        <v>6.0270967310671075</v>
+      </c>
+      <c r="U18" s="4">
         <f t="shared" si="7"/>
-        <v>14.26</v>
-      </c>
-      <c r="P18">
-        <f t="shared" si="3"/>
-        <v>9.8999999999999986</v>
-      </c>
-      <c r="Q18">
-        <f t="shared" si="4"/>
-        <v>10.479999999999999</v>
-      </c>
-      <c r="R18" s="4">
-        <f t="shared" si="5"/>
-        <v>8.9749120996731335</v>
-      </c>
-      <c r="S18" s="4">
-        <f t="shared" si="6"/>
-        <v>6.0270967310671075</v>
-      </c>
-      <c r="T18" s="4">
-        <f t="shared" si="8"/>
         <v>35.134709089637553</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>46028.691666666666</v>
       </c>
@@ -2005,49 +2039,53 @@
         <v>12.09</v>
       </c>
       <c r="H19">
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>40.532312299018905</v>
       </c>
       <c r="I19">
+        <v>0</v>
+      </c>
+      <c r="J19">
         <v>41</v>
       </c>
-      <c r="J19">
+      <c r="K19">
         <v>25.2</v>
       </c>
-      <c r="K19">
+      <c r="L19">
         <v>33.6</v>
       </c>
-      <c r="L19">
-        <v>0</v>
-      </c>
       <c r="M19">
+        <v>0</v>
+      </c>
+      <c r="N19">
         <v>55.853999999999999</v>
       </c>
-      <c r="O19">
+      <c r="P19">
+        <f t="shared" si="6"/>
+        <v>14.3</v>
+      </c>
+      <c r="Q19">
+        <f t="shared" si="2"/>
+        <v>9.84</v>
+      </c>
+      <c r="R19">
+        <f t="shared" si="3"/>
+        <v>12.04</v>
+      </c>
+      <c r="S19" s="4">
+        <f t="shared" si="4"/>
+        <v>9.0000871686764263</v>
+      </c>
+      <c r="T19" s="4">
+        <f t="shared" si="5"/>
+        <v>5.990568872090944</v>
+      </c>
+      <c r="U19" s="4">
         <f t="shared" si="7"/>
-        <v>14.3</v>
-      </c>
-      <c r="P19">
-        <f t="shared" si="3"/>
-        <v>9.84</v>
-      </c>
-      <c r="Q19">
-        <f t="shared" si="4"/>
-        <v>12.04</v>
-      </c>
-      <c r="R19" s="4">
-        <f t="shared" si="5"/>
-        <v>9.0000871686764263</v>
-      </c>
-      <c r="S19" s="4">
-        <f t="shared" si="6"/>
-        <v>5.990568872090944</v>
-      </c>
-      <c r="T19" s="4">
-        <f t="shared" si="8"/>
         <v>40.364684870156125</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>46028.692361111112</v>
       </c>
@@ -2070,49 +2108,53 @@
         <v>13.58</v>
       </c>
       <c r="H20">
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>45.52760967912959</v>
       </c>
       <c r="I20">
+        <v>0</v>
+      </c>
+      <c r="J20">
         <v>39.299999999999997</v>
       </c>
-      <c r="J20">
+      <c r="K20">
         <v>24.2</v>
       </c>
-      <c r="K20">
+      <c r="L20">
         <v>36.299999999999997</v>
       </c>
-      <c r="L20">
-        <v>0</v>
-      </c>
       <c r="M20">
+        <v>0</v>
+      </c>
+      <c r="N20">
         <v>58.192999999999998</v>
       </c>
-      <c r="O20">
+      <c r="P20">
+        <f t="shared" si="6"/>
+        <v>14.280000000000001</v>
+      </c>
+      <c r="Q20">
+        <f t="shared" si="2"/>
+        <v>9.82</v>
+      </c>
+      <c r="R20">
+        <f t="shared" si="3"/>
+        <v>13.53</v>
+      </c>
+      <c r="S20" s="4">
+        <f t="shared" si="4"/>
+        <v>8.9874996341747799</v>
+      </c>
+      <c r="T20" s="4">
+        <f t="shared" si="5"/>
+        <v>5.9783929190988889</v>
+      </c>
+      <c r="U20" s="4">
         <f t="shared" si="7"/>
-        <v>14.280000000000001</v>
-      </c>
-      <c r="P20">
-        <f t="shared" si="3"/>
-        <v>9.82</v>
-      </c>
-      <c r="Q20">
-        <f t="shared" si="4"/>
-        <v>13.53</v>
-      </c>
-      <c r="R20" s="4">
-        <f t="shared" si="5"/>
-        <v>8.9874996341747799</v>
-      </c>
-      <c r="S20" s="4">
-        <f t="shared" si="6"/>
-        <v>5.9783929190988889</v>
-      </c>
-      <c r="T20" s="4">
-        <f t="shared" si="8"/>
         <v>45.35998225026681</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>46028.693055555559</v>
       </c>
@@ -2135,49 +2177,53 @@
         <v>14.53</v>
       </c>
       <c r="H21">
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>48.712530827522301</v>
       </c>
       <c r="I21">
+        <v>0</v>
+      </c>
+      <c r="J21">
         <v>38.4</v>
       </c>
-      <c r="J21">
+      <c r="K21">
         <v>23.6</v>
       </c>
-      <c r="K21">
+      <c r="L21">
         <v>37.9</v>
       </c>
-      <c r="L21">
-        <v>0</v>
-      </c>
       <c r="M21">
+        <v>0</v>
+      </c>
+      <c r="N21">
         <v>59.667000000000002</v>
       </c>
-      <c r="O21">
+      <c r="P21">
+        <f t="shared" si="6"/>
+        <v>14.34</v>
+      </c>
+      <c r="Q21">
+        <f t="shared" si="2"/>
+        <v>9.86</v>
+      </c>
+      <c r="R21">
+        <f t="shared" si="3"/>
+        <v>14.479999999999999</v>
+      </c>
+      <c r="S21" s="4">
+        <f t="shared" si="4"/>
+        <v>9.0252622376797156</v>
+      </c>
+      <c r="T21" s="4">
+        <f t="shared" si="5"/>
+        <v>6.0027448250829982</v>
+      </c>
+      <c r="U21" s="4">
         <f t="shared" si="7"/>
-        <v>14.34</v>
-      </c>
-      <c r="P21">
-        <f t="shared" si="3"/>
-        <v>9.86</v>
-      </c>
-      <c r="Q21">
-        <f t="shared" si="4"/>
-        <v>14.479999999999999</v>
-      </c>
-      <c r="R21" s="4">
-        <f t="shared" si="5"/>
-        <v>9.0252622376797156</v>
-      </c>
-      <c r="S21" s="4">
-        <f t="shared" si="6"/>
-        <v>6.0027448250829982</v>
-      </c>
-      <c r="T21" s="4">
-        <f t="shared" si="8"/>
         <v>48.544903398659528</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>46028.693749999999</v>
       </c>
@@ -2200,49 +2246,53 @@
         <v>14.53</v>
       </c>
       <c r="H22">
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>48.712530827522301</v>
       </c>
       <c r="I22">
+        <v>0</v>
+      </c>
+      <c r="J22">
         <v>49</v>
       </c>
-      <c r="J22">
+      <c r="K22">
         <v>6551</v>
       </c>
-      <c r="K22">
+      <c r="L22">
         <v>48.3</v>
       </c>
-      <c r="L22">
-        <v>0</v>
-      </c>
       <c r="M22">
+        <v>0</v>
+      </c>
+      <c r="N22">
         <v>44.317</v>
       </c>
-      <c r="O22">
+      <c r="P22">
+        <f t="shared" si="6"/>
+        <v>14.32</v>
+      </c>
+      <c r="Q22">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="R22">
+        <f t="shared" si="3"/>
+        <v>14.479999999999999</v>
+      </c>
+      <c r="S22" s="4">
+        <f t="shared" si="4"/>
+        <v>9.012674703178071</v>
+      </c>
+      <c r="T22" s="4">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="U22" s="4">
         <f t="shared" si="7"/>
-        <v>14.32</v>
-      </c>
-      <c r="P22">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="Q22">
-        <f t="shared" si="4"/>
-        <v>14.479999999999999</v>
-      </c>
-      <c r="R22" s="4">
-        <f t="shared" si="5"/>
-        <v>9.012674703178071</v>
-      </c>
-      <c r="S22" s="4">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="T22" s="4">
-        <f t="shared" si="8"/>
         <v>48.544903398659528</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>46028.694444444445</v>
       </c>
@@ -2265,49 +2315,53 @@
         <v>10.93</v>
       </c>
       <c r="H23">
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>36.643355949402533</v>
       </c>
       <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23">
         <v>42.4</v>
       </c>
-      <c r="J23">
+      <c r="K23">
         <v>26</v>
       </c>
-      <c r="K23">
+      <c r="L23">
         <v>31.4</v>
       </c>
-      <c r="L23">
-        <v>0</v>
-      </c>
       <c r="M23">
+        <v>0</v>
+      </c>
+      <c r="N23">
         <v>54.073999999999998</v>
       </c>
-      <c r="O23">
+      <c r="P23">
+        <f t="shared" si="6"/>
+        <v>14.35</v>
+      </c>
+      <c r="Q23">
+        <f t="shared" si="2"/>
+        <v>9.86</v>
+      </c>
+      <c r="R23">
+        <f t="shared" si="3"/>
+        <v>10.879999999999999</v>
+      </c>
+      <c r="S23" s="4">
+        <f t="shared" si="4"/>
+        <v>9.0315560049305379</v>
+      </c>
+      <c r="T23" s="4">
+        <f t="shared" si="5"/>
+        <v>6.0027448250829982</v>
+      </c>
+      <c r="U23" s="4">
         <f t="shared" si="7"/>
-        <v>14.35</v>
-      </c>
-      <c r="P23">
-        <f t="shared" si="3"/>
-        <v>9.86</v>
-      </c>
-      <c r="Q23">
-        <f t="shared" si="4"/>
-        <v>10.879999999999999</v>
-      </c>
-      <c r="R23" s="4">
-        <f t="shared" si="5"/>
-        <v>9.0315560049305379</v>
-      </c>
-      <c r="S23" s="4">
-        <f t="shared" si="6"/>
-        <v>6.0027448250829982</v>
-      </c>
-      <c r="T23" s="4">
-        <f t="shared" si="8"/>
         <v>36.475728520539754</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>46028.694444444445</v>
       </c>
@@ -2330,49 +2384,53 @@
         <v>8.33</v>
       </c>
       <c r="H24">
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>27.926729648538252</v>
       </c>
       <c r="I24">
+        <v>0</v>
+      </c>
+      <c r="J24">
         <v>45.8</v>
       </c>
-      <c r="J24">
+      <c r="K24">
         <v>28.2</v>
       </c>
-      <c r="K24">
+      <c r="L24">
         <v>25.9</v>
       </c>
-      <c r="L24">
-        <v>0</v>
-      </c>
       <c r="M24">
+        <v>0</v>
+      </c>
+      <c r="N24">
         <v>50.021000000000001</v>
       </c>
-      <c r="O24">
+      <c r="P24">
+        <f t="shared" si="6"/>
+        <v>14.25</v>
+      </c>
+      <c r="Q24">
+        <f t="shared" si="2"/>
+        <v>9.86</v>
+      </c>
+      <c r="R24">
+        <f t="shared" si="3"/>
+        <v>8.2799999999999994</v>
+      </c>
+      <c r="S24" s="4">
+        <f t="shared" si="4"/>
+        <v>8.9686183324223112</v>
+      </c>
+      <c r="T24" s="4">
+        <f t="shared" si="5"/>
+        <v>6.0027448250829982</v>
+      </c>
+      <c r="U24" s="4">
         <f t="shared" si="7"/>
-        <v>14.25</v>
-      </c>
-      <c r="P24">
-        <f t="shared" si="3"/>
-        <v>9.86</v>
-      </c>
-      <c r="Q24">
-        <f t="shared" si="4"/>
-        <v>8.2799999999999994</v>
-      </c>
-      <c r="R24" s="4">
-        <f t="shared" si="5"/>
-        <v>8.9686183324223112</v>
-      </c>
-      <c r="S24" s="4">
-        <f t="shared" si="6"/>
-        <v>6.0027448250829982</v>
-      </c>
-      <c r="T24" s="4">
-        <f t="shared" si="8"/>
         <v>27.759102219675476</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>46028.695138888892</v>
       </c>
@@ -2395,49 +2453,53 @@
         <v>5.68</v>
       </c>
       <c r="H25">
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>19.042475918811196</v>
       </c>
       <c r="I25">
+        <v>0</v>
+      </c>
+      <c r="J25">
         <v>49.9</v>
       </c>
-      <c r="J25">
+      <c r="K25">
         <v>30.7</v>
       </c>
-      <c r="K25">
+      <c r="L25">
         <v>19.2</v>
       </c>
-      <c r="L25">
-        <v>0</v>
-      </c>
       <c r="M25">
+        <v>0</v>
+      </c>
+      <c r="N25">
         <v>45.898000000000003</v>
       </c>
-      <c r="O25">
+      <c r="P25">
+        <f t="shared" si="6"/>
+        <v>14.31</v>
+      </c>
+      <c r="Q25">
+        <f t="shared" si="2"/>
+        <v>9.86</v>
+      </c>
+      <c r="R25">
+        <f t="shared" si="3"/>
+        <v>5.63</v>
+      </c>
+      <c r="S25" s="4">
+        <f t="shared" si="4"/>
+        <v>9.0063809359272486</v>
+      </c>
+      <c r="T25" s="4">
+        <f t="shared" si="5"/>
+        <v>6.0027448250829982</v>
+      </c>
+      <c r="U25" s="4">
         <f t="shared" si="7"/>
-        <v>14.31</v>
-      </c>
-      <c r="P25">
-        <f t="shared" si="3"/>
-        <v>9.86</v>
-      </c>
-      <c r="Q25">
-        <f t="shared" si="4"/>
-        <v>5.63</v>
-      </c>
-      <c r="R25" s="4">
-        <f t="shared" si="5"/>
-        <v>9.0063809359272486</v>
-      </c>
-      <c r="S25" s="4">
-        <f t="shared" si="6"/>
-        <v>6.0027448250829982</v>
-      </c>
-      <c r="T25" s="4">
-        <f t="shared" si="8"/>
         <v>18.874848489948423</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>46028.695833333331</v>
       </c>
@@ -2460,49 +2522,53 @@
         <v>3.33</v>
       </c>
       <c r="H26">
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>11.163986762260789</v>
       </c>
       <c r="I26">
+        <v>0</v>
+      </c>
+      <c r="J26">
         <v>54.2</v>
       </c>
-      <c r="J26">
+      <c r="K26">
         <v>33.4</v>
       </c>
-      <c r="K26">
+      <c r="L26">
         <v>12.2</v>
       </c>
-      <c r="L26">
-        <v>0</v>
-      </c>
       <c r="M26">
+        <v>0</v>
+      </c>
+      <c r="N26">
         <v>42.238999999999997</v>
       </c>
-      <c r="O26">
+      <c r="P26">
+        <f t="shared" si="6"/>
+        <v>14.32</v>
+      </c>
+      <c r="Q26">
+        <f t="shared" si="2"/>
+        <v>9.84</v>
+      </c>
+      <c r="R26">
+        <f t="shared" si="3"/>
+        <v>3.2800000000000002</v>
+      </c>
+      <c r="S26" s="4">
+        <f t="shared" si="4"/>
+        <v>9.012674703178071</v>
+      </c>
+      <c r="T26" s="4">
+        <f t="shared" si="5"/>
+        <v>5.990568872090944</v>
+      </c>
+      <c r="U26" s="4">
         <f t="shared" si="7"/>
-        <v>14.32</v>
-      </c>
-      <c r="P26">
-        <f t="shared" si="3"/>
-        <v>9.84</v>
-      </c>
-      <c r="Q26">
-        <f t="shared" si="4"/>
-        <v>3.2800000000000002</v>
-      </c>
-      <c r="R26" s="4">
-        <f t="shared" si="5"/>
-        <v>9.012674703178071</v>
-      </c>
-      <c r="S26" s="4">
-        <f t="shared" si="6"/>
-        <v>5.990568872090944</v>
-      </c>
-      <c r="T26" s="4">
-        <f t="shared" si="8"/>
         <v>10.996359333398015</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>46028.695833333331</v>
       </c>
@@ -2525,49 +2591,53 @@
         <v>1.58</v>
       </c>
       <c r="H27">
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>5.2970267520636778</v>
       </c>
       <c r="I27">
+        <v>0</v>
+      </c>
+      <c r="J27">
         <v>58</v>
       </c>
-      <c r="J27">
+      <c r="K27">
         <v>35.700000000000003</v>
       </c>
-      <c r="K27">
+      <c r="L27">
         <v>6.2</v>
       </c>
-      <c r="L27">
-        <v>0</v>
-      </c>
       <c r="M27">
+        <v>0</v>
+      </c>
+      <c r="N27">
         <v>39.518000000000001</v>
       </c>
-      <c r="O27">
+      <c r="P27">
+        <f t="shared" si="6"/>
+        <v>14.31</v>
+      </c>
+      <c r="Q27">
+        <f t="shared" si="2"/>
+        <v>9.86</v>
+      </c>
+      <c r="R27">
+        <f t="shared" si="3"/>
+        <v>1.53</v>
+      </c>
+      <c r="S27" s="4">
+        <f t="shared" si="4"/>
+        <v>9.0063809359272486</v>
+      </c>
+      <c r="T27" s="4">
+        <f t="shared" si="5"/>
+        <v>6.0027448250829982</v>
+      </c>
+      <c r="U27" s="4">
         <f t="shared" si="7"/>
-        <v>14.31</v>
-      </c>
-      <c r="P27">
-        <f t="shared" si="3"/>
-        <v>9.86</v>
-      </c>
-      <c r="Q27">
-        <f t="shared" si="4"/>
-        <v>1.53</v>
-      </c>
-      <c r="R27" s="4">
-        <f t="shared" si="5"/>
-        <v>9.0063809359272486</v>
-      </c>
-      <c r="S27" s="4">
-        <f t="shared" si="6"/>
-        <v>6.0027448250829982</v>
-      </c>
-      <c r="T27" s="4">
-        <f t="shared" si="8"/>
         <v>5.1293993232009036</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>46028.696527777778</v>
       </c>
@@ -2590,49 +2660,53 @@
         <v>0.6</v>
       </c>
       <c r="H28">
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>2.0115291463532952</v>
       </c>
       <c r="I28">
+        <v>0</v>
+      </c>
+      <c r="J28">
         <v>60.3</v>
       </c>
-      <c r="J28">
+      <c r="K28">
         <v>37.1</v>
       </c>
-      <c r="K28">
+      <c r="L28">
         <v>2.4</v>
       </c>
-      <c r="L28">
-        <v>0</v>
-      </c>
       <c r="M28">
+        <v>0</v>
+      </c>
+      <c r="N28">
         <v>37.970999999999997</v>
       </c>
-      <c r="O28">
+      <c r="P28">
+        <f t="shared" si="6"/>
+        <v>14.25</v>
+      </c>
+      <c r="Q28">
+        <f t="shared" si="2"/>
+        <v>9.8099999999999987</v>
+      </c>
+      <c r="R28">
+        <f t="shared" si="3"/>
+        <v>0.54999999999999993</v>
+      </c>
+      <c r="S28" s="4">
+        <f t="shared" si="4"/>
+        <v>8.9686183324223112</v>
+      </c>
+      <c r="T28" s="4">
+        <f t="shared" si="5"/>
+        <v>5.9723049426028609</v>
+      </c>
+      <c r="U28" s="4">
         <f t="shared" si="7"/>
-        <v>14.25</v>
-      </c>
-      <c r="P28">
-        <f t="shared" si="3"/>
-        <v>9.8099999999999987</v>
-      </c>
-      <c r="Q28">
-        <f t="shared" si="4"/>
-        <v>0.54999999999999993</v>
-      </c>
-      <c r="R28" s="4">
-        <f t="shared" si="5"/>
-        <v>8.9686183324223112</v>
-      </c>
-      <c r="S28" s="4">
-        <f t="shared" si="6"/>
-        <v>5.9723049426028609</v>
-      </c>
-      <c r="T28" s="4">
-        <f t="shared" si="8"/>
         <v>1.8439017174905206</v>
       </c>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>46028.696527777778</v>
       </c>
@@ -2655,49 +2729,53 @@
         <v>0.06</v>
       </c>
       <c r="H29">
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>0.20115291463532953</v>
       </c>
       <c r="I29">
+        <v>0</v>
+      </c>
+      <c r="J29">
         <v>61.7</v>
       </c>
-      <c r="J29">
+      <c r="K29">
         <v>38</v>
       </c>
-      <c r="K29">
+      <c r="L29">
         <v>0.2</v>
       </c>
-      <c r="L29">
-        <v>0</v>
-      </c>
       <c r="M29">
+        <v>0</v>
+      </c>
+      <c r="N29">
         <v>37.152999999999999</v>
       </c>
-      <c r="O29">
+      <c r="P29">
+        <f t="shared" si="6"/>
+        <v>14.31</v>
+      </c>
+      <c r="Q29">
+        <f t="shared" si="2"/>
+        <v>9.8299999999999983</v>
+      </c>
+      <c r="R29">
+        <f t="shared" si="3"/>
+        <v>9.999999999999995E-3</v>
+      </c>
+      <c r="S29" s="4">
+        <f t="shared" si="4"/>
+        <v>9.0063809359272486</v>
+      </c>
+      <c r="T29" s="4">
+        <f t="shared" si="5"/>
+        <v>5.9844808955949151</v>
+      </c>
+      <c r="U29" s="4">
         <f t="shared" si="7"/>
-        <v>14.31</v>
-      </c>
-      <c r="P29">
-        <f t="shared" si="3"/>
-        <v>9.8299999999999983</v>
-      </c>
-      <c r="Q29">
-        <f t="shared" si="4"/>
-        <v>9.999999999999995E-3</v>
-      </c>
-      <c r="R29" s="4">
-        <f t="shared" si="5"/>
-        <v>9.0063809359272486</v>
-      </c>
-      <c r="S29" s="4">
-        <f t="shared" si="6"/>
-        <v>5.9844808955949151</v>
-      </c>
-      <c r="T29" s="4">
-        <f t="shared" si="8"/>
         <v>3.352548577255491E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>46028.697222222225</v>
       </c>
@@ -2720,56 +2798,60 @@
         <v>0.06</v>
       </c>
       <c r="H30">
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>0.20115291463532953</v>
       </c>
       <c r="I30">
+        <v>0</v>
+      </c>
+      <c r="J30">
         <v>34.1</v>
       </c>
-      <c r="J30">
+      <c r="K30">
         <v>6492.9</v>
       </c>
-      <c r="K30">
+      <c r="L30">
         <v>5</v>
       </c>
-      <c r="L30">
-        <v>0</v>
-      </c>
       <c r="M30">
+        <v>0</v>
+      </c>
+      <c r="N30">
         <v>-0.438</v>
       </c>
-      <c r="O30">
+      <c r="P30">
+        <f t="shared" si="6"/>
+        <v>1.0000000000000009E-2</v>
+      </c>
+      <c r="Q30">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="R30">
+        <f t="shared" si="3"/>
+        <v>9.999999999999995E-3</v>
+      </c>
+      <c r="S30" s="4">
+        <f t="shared" si="4"/>
+        <v>6.2937672508226808E-3</v>
+      </c>
+      <c r="T30" s="4">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="U30" s="4">
         <f t="shared" si="7"/>
-        <v>1.0000000000000009E-2</v>
-      </c>
-      <c r="P30">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="Q30">
-        <f t="shared" si="4"/>
-        <v>9.999999999999995E-3</v>
-      </c>
-      <c r="R30" s="4">
-        <f t="shared" si="5"/>
-        <v>6.2937672508226808E-3</v>
-      </c>
-      <c r="S30" s="4">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="T30" s="4">
-        <f t="shared" si="8"/>
         <v>3.352548577255491E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="33" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="33" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B33" s="8" t="str">
         <f>B9</f>
         <v>Bucket1</v>
       </c>
       <c r="C33" s="9" t="str">
-        <f>R9</f>
+        <f>S9</f>
         <v>Ch1_Load</v>
       </c>
       <c r="D33" s="9" t="s">
@@ -2780,25 +2862,26 @@
         <v>Bucket2</v>
       </c>
       <c r="F33" s="9" t="str">
-        <f>S9</f>
+        <f>T9</f>
         <v>Ch2_Load</v>
       </c>
       <c r="G33" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="H33" s="9" t="str">
+      <c r="H33" s="9"/>
+      <c r="I33" s="9" t="str">
         <f>D9</f>
         <v>Bucket3</v>
       </c>
-      <c r="I33" s="9" t="str">
-        <f t="shared" ref="I33" si="9">T9</f>
+      <c r="J33" s="9" t="str">
+        <f t="shared" ref="J33" si="8">U9</f>
         <v>Ch3_Load</v>
       </c>
-      <c r="J33" s="10" t="s">
+      <c r="K33" s="10" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="34" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B34" s="11" t="s">
         <v>37</v>
       </c>
@@ -2817,29 +2900,30 @@
       <c r="G34" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="H34" s="12" t="s">
-        <v>37</v>
-      </c>
+      <c r="H34" s="12"/>
       <c r="I34" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="J34" s="13" t="s">
+      <c r="J34" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="M34" s="14" t="s">
+      <c r="K34" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="N34" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="N34" s="14" t="s">
+      <c r="O34" s="14" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="35" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B35" s="6">
         <f>B11*453.59237</f>
         <v>0</v>
       </c>
       <c r="C35" s="6">
-        <f t="shared" ref="C35:C54" si="10">R11*453.59237</f>
+        <f t="shared" ref="C35:C54" si="9">S11*453.59237</f>
         <v>0</v>
       </c>
       <c r="D35" s="3">
@@ -2847,52 +2931,53 @@
         <v>0</v>
       </c>
       <c r="E35" s="6">
-        <f t="shared" ref="E35:E54" si="11">C11*453.59237</f>
+        <f t="shared" ref="E35:E54" si="10">C11*453.59237</f>
         <v>0</v>
       </c>
       <c r="F35" s="6">
-        <f t="shared" ref="F35:F54" si="12">S11*453.59237</f>
+        <f t="shared" ref="F35:F54" si="11">T11*453.59237</f>
         <v>0</v>
       </c>
       <c r="G35" s="7">
         <f>F35-E35</f>
         <v>0</v>
       </c>
-      <c r="H35" s="6">
-        <f t="shared" ref="H35:H54" si="13">D11*453.59237</f>
-        <v>0</v>
-      </c>
+      <c r="H35" s="7"/>
       <c r="I35" s="6">
-        <f t="shared" ref="I35:I50" si="14">T11*453.59237</f>
-        <v>0</v>
-      </c>
-      <c r="J35" s="7">
-        <f>I35-H35</f>
-        <v>0</v>
-      </c>
-      <c r="L35" s="3">
-        <f>G11*$N$35+$O$35</f>
+        <f t="shared" ref="I35:I54" si="12">D11*453.59237</f>
+        <v>0</v>
+      </c>
+      <c r="J35" s="6">
+        <f t="shared" ref="J35:J50" si="13">U11*453.59237</f>
+        <v>0</v>
+      </c>
+      <c r="K35" s="7">
+        <f>J35-I35</f>
+        <v>0</v>
+      </c>
+      <c r="M35" s="3">
+        <f>G11*$O$35+$P$35</f>
         <v>-10.0193861542501</v>
       </c>
-      <c r="M35" s="3">
-        <f>ABS(L35-H35)</f>
+      <c r="N35" s="3">
+        <f>ABS(M35-I35)</f>
         <v>10.0193861542501</v>
       </c>
-      <c r="N35" cm="1">
-        <f t="array" ref="N35:O35">LINEST(H35:H54,G11:G30)</f>
+      <c r="O35" cm="1">
+        <f t="array" ref="O35:P35">LINEST(I35:I54,G11:G30)</f>
         <v>1507.3123323796999</v>
       </c>
-      <c r="O35">
+      <c r="P35">
         <v>-85.385002773235101</v>
       </c>
     </row>
-    <row r="36" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B36" s="5">
-        <f t="shared" ref="B36:B54" si="15">B12*453.59237</f>
+        <f t="shared" ref="B36:B54" si="14">B12*453.59237</f>
         <v>4064.1876352000004</v>
       </c>
       <c r="C36" s="5">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>4076.6612594394715</v>
       </c>
       <c r="D36" s="3">
@@ -2900,867 +2985,886 @@
         <v>12.473624239471064</v>
       </c>
       <c r="E36" s="5">
+        <f t="shared" si="10"/>
+        <v>2712.4823726000004</v>
+      </c>
+      <c r="F36" s="5">
         <f t="shared" si="11"/>
-        <v>2712.4823726000004</v>
-      </c>
-      <c r="F36" s="5">
-        <f t="shared" si="12"/>
         <v>2722.7992517146326</v>
       </c>
       <c r="G36" s="5">
         <f>ABS(F36-E36)</f>
         <v>10.316879114632229</v>
       </c>
-      <c r="H36" s="5">
+      <c r="H36" s="5"/>
+      <c r="I36" s="5">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J36" s="5">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="I36" s="5">
+      <c r="K36" s="5">
+        <f>ABS(J36-I36)</f>
+        <v>0</v>
+      </c>
+      <c r="M36" s="3">
+        <f t="shared" ref="M36:M54" si="15">G12*$O$35+$P$35</f>
+        <v>-10.0193861542501</v>
+      </c>
+      <c r="N36" s="3">
+        <f t="shared" ref="N36:N54" si="16">ABS(M36-I36)</f>
+        <v>10.0193861542501</v>
+      </c>
+    </row>
+    <row r="37" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B37" s="5">
         <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="J36" s="5">
-        <f>ABS(I36-H36)</f>
-        <v>0</v>
-      </c>
-      <c r="L36" s="3">
-        <f t="shared" ref="L36:L54" si="16">G12*$N$35+$O$35</f>
-        <v>-10.0193861542501</v>
-      </c>
-      <c r="M36" s="3">
-        <f t="shared" ref="M36:M54" si="17">ABS(L36-H36)</f>
-        <v>10.0193861542501</v>
-      </c>
-    </row>
-    <row r="37" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B37" s="5">
+        <v>4064.1876352000004</v>
+      </c>
+      <c r="C37" s="5">
+        <f t="shared" si="9"/>
+        <v>4068.0968450288842</v>
+      </c>
+      <c r="D37" s="3">
+        <f t="shared" ref="D37:D54" si="17">ABS(C37-B37)</f>
+        <v>3.9092098288838315</v>
+      </c>
+      <c r="E37" s="5">
+        <f t="shared" si="10"/>
+        <v>2712.4823726000004</v>
+      </c>
+      <c r="F37" s="5">
+        <f t="shared" si="11"/>
+        <v>2733.8450904639822</v>
+      </c>
+      <c r="G37" s="5">
+        <f t="shared" ref="G37:G54" si="18">ABS(F37-E37)</f>
+        <v>21.362717863981743</v>
+      </c>
+      <c r="H37" s="5"/>
+      <c r="I37" s="5">
+        <f t="shared" si="12"/>
+        <v>802.85849489999998</v>
+      </c>
+      <c r="J37" s="5">
+        <f t="shared" si="13"/>
+        <v>821.17284553662125</v>
+      </c>
+      <c r="K37" s="5">
+        <f t="shared" ref="K37:K54" si="19">ABS(J37-I37)</f>
+        <v>18.31435063662127</v>
+      </c>
+      <c r="M37" s="3">
         <f t="shared" si="15"/>
+        <v>803.92927333078785</v>
+      </c>
+      <c r="N37" s="3">
+        <f t="shared" si="16"/>
+        <v>1.0707784307878683</v>
+      </c>
+    </row>
+    <row r="38" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B38" s="5">
+        <f t="shared" si="14"/>
         <v>4064.1876352000004</v>
       </c>
-      <c r="C37" s="5">
+      <c r="C38" s="5">
+        <f t="shared" si="9"/>
+        <v>4082.3708690465301</v>
+      </c>
+      <c r="D38" s="3">
+        <f t="shared" si="17"/>
+        <v>18.183233846529674</v>
+      </c>
+      <c r="E38" s="5">
         <f t="shared" si="10"/>
+        <v>2712.4823726000004</v>
+      </c>
+      <c r="F38" s="5">
+        <f t="shared" si="11"/>
+        <v>2744.8909292133321</v>
+      </c>
+      <c r="G38" s="5">
+        <f t="shared" si="18"/>
+        <v>32.408556613331712</v>
+      </c>
+      <c r="H38" s="5"/>
+      <c r="I38" s="5">
+        <f t="shared" si="12"/>
+        <v>2345.0725529000001</v>
+      </c>
+      <c r="J38" s="5">
+        <f t="shared" si="13"/>
+        <v>2357.0702047810428</v>
+      </c>
+      <c r="K38" s="5">
+        <f t="shared" si="19"/>
+        <v>11.997651881042657</v>
+      </c>
+      <c r="M38" s="3">
+        <f t="shared" si="15"/>
+        <v>2326.3147290342849</v>
+      </c>
+      <c r="N38" s="3">
+        <f t="shared" si="16"/>
+        <v>18.757823865715181</v>
+      </c>
+    </row>
+    <row r="39" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B39" s="5">
+        <f t="shared" si="14"/>
+        <v>4064.1876352000004</v>
+      </c>
+      <c r="C39" s="5">
+        <f t="shared" si="9"/>
+        <v>4090.9352834571168</v>
+      </c>
+      <c r="D39" s="3">
+        <f t="shared" si="17"/>
+        <v>26.747648257116452</v>
+      </c>
+      <c r="E39" s="5">
+        <f t="shared" si="10"/>
+        <v>2712.4823726000004</v>
+      </c>
+      <c r="F39" s="5">
+        <f t="shared" si="11"/>
+        <v>2714.5148726526204</v>
+      </c>
+      <c r="G39" s="5">
+        <f t="shared" si="18"/>
+        <v>2.0325000526199801</v>
+      </c>
+      <c r="H39" s="5"/>
+      <c r="I39" s="5">
+        <f t="shared" si="12"/>
+        <v>5102.9141625000002</v>
+      </c>
+      <c r="J39" s="5">
+        <f t="shared" si="13"/>
+        <v>5155.1406414243447</v>
+      </c>
+      <c r="K39" s="5">
+        <f t="shared" si="19"/>
+        <v>52.226478924344519</v>
+      </c>
+      <c r="M39" s="3">
+        <f t="shared" si="15"/>
+        <v>5099.7694206129327</v>
+      </c>
+      <c r="N39" s="3">
+        <f t="shared" si="16"/>
+        <v>3.1447418870675392</v>
+      </c>
+    </row>
+    <row r="40" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B40" s="5">
+        <f t="shared" si="14"/>
+        <v>4064.1876352000004</v>
+      </c>
+      <c r="C40" s="5">
+        <f t="shared" si="9"/>
+        <v>4082.3708690465301</v>
+      </c>
+      <c r="D40" s="3">
+        <f t="shared" si="17"/>
+        <v>18.183233846529674</v>
+      </c>
+      <c r="E40" s="5">
+        <f t="shared" si="10"/>
+        <v>2712.4823726000004</v>
+      </c>
+      <c r="F40" s="5">
+        <f t="shared" si="11"/>
+        <v>2722.7992517146326</v>
+      </c>
+      <c r="G40" s="5">
+        <f t="shared" si="18"/>
+        <v>10.316879114632229</v>
+      </c>
+      <c r="H40" s="5"/>
+      <c r="I40" s="5">
+        <f t="shared" si="12"/>
+        <v>8600.1113352000011</v>
+      </c>
+      <c r="J40" s="5">
+        <f t="shared" si="13"/>
+        <v>8683.1424963224217</v>
+      </c>
+      <c r="K40" s="5">
+        <f t="shared" si="19"/>
+        <v>83.031161122420599</v>
+      </c>
+      <c r="M40" s="3">
+        <f t="shared" si="15"/>
+        <v>8596.7340317338367</v>
+      </c>
+      <c r="N40" s="3">
+        <f t="shared" si="16"/>
+        <v>3.3773034661644488</v>
+      </c>
+    </row>
+    <row r="41" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B41" s="5">
+        <f t="shared" si="14"/>
+        <v>4064.1876352000004</v>
+      </c>
+      <c r="C41" s="5">
+        <f t="shared" si="9"/>
+        <v>4079.5160642430005</v>
+      </c>
+      <c r="D41" s="3">
+        <f t="shared" si="17"/>
+        <v>15.328429043000142</v>
+      </c>
+      <c r="E41" s="5">
+        <f t="shared" si="10"/>
+        <v>2712.4823726000004</v>
+      </c>
+      <c r="F41" s="5">
+        <f t="shared" si="11"/>
+        <v>2720.0377920272958</v>
+      </c>
+      <c r="G41" s="5">
+        <f t="shared" si="18"/>
+        <v>7.5554194272954192</v>
+      </c>
+      <c r="H41" s="5"/>
+      <c r="I41" s="5">
+        <f t="shared" si="12"/>
+        <v>12451.1105565</v>
+      </c>
+      <c r="J41" s="5">
+        <f t="shared" si="13"/>
+        <v>12560.90315580091</v>
+      </c>
+      <c r="K41" s="5">
+        <f t="shared" si="19"/>
+        <v>109.7925993009103</v>
+      </c>
+      <c r="M41" s="3">
+        <f t="shared" si="15"/>
+        <v>12440.380479302072</v>
+      </c>
+      <c r="N41" s="3">
+        <f t="shared" si="16"/>
+        <v>10.73007719792804</v>
+      </c>
+    </row>
+    <row r="42" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B42" s="5">
+        <f t="shared" si="14"/>
+        <v>4064.1876352000004</v>
+      </c>
+      <c r="C42" s="5">
+        <f t="shared" si="9"/>
+        <v>4070.9516498324128</v>
+      </c>
+      <c r="D42" s="3">
+        <f t="shared" si="17"/>
+        <v>6.7640146324124544</v>
+      </c>
+      <c r="E42" s="5">
+        <f t="shared" si="10"/>
+        <v>2712.4823726000004</v>
+      </c>
+      <c r="F42" s="5">
+        <f t="shared" si="11"/>
+        <v>2733.8450904639822</v>
+      </c>
+      <c r="G42" s="5">
+        <f t="shared" si="18"/>
+        <v>21.362717863981743</v>
+      </c>
+      <c r="H42" s="5"/>
+      <c r="I42" s="5">
+        <f t="shared" si="12"/>
+        <v>15794.086323400001</v>
+      </c>
+      <c r="J42" s="5">
+        <f t="shared" si="13"/>
+        <v>15936.83596522924</v>
+      </c>
+      <c r="K42" s="5">
+        <f t="shared" si="19"/>
+        <v>142.74964182923941</v>
+      </c>
+      <c r="M42" s="3">
+        <f t="shared" si="15"/>
+        <v>15786.613857185004</v>
+      </c>
+      <c r="N42" s="3">
+        <f t="shared" si="16"/>
+        <v>7.4724662149965297</v>
+      </c>
+    </row>
+    <row r="43" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B43" s="5">
+        <f t="shared" si="14"/>
+        <v>4064.1876352000004</v>
+      </c>
+      <c r="C43" s="5">
+        <f t="shared" si="9"/>
+        <v>4082.3708690465301</v>
+      </c>
+      <c r="D43" s="3">
+        <f t="shared" si="17"/>
+        <v>18.183233846529674</v>
+      </c>
+      <c r="E43" s="5">
+        <f t="shared" si="10"/>
+        <v>2712.4823726000004</v>
+      </c>
+      <c r="F43" s="5">
+        <f t="shared" si="11"/>
+        <v>2717.2763323399581</v>
+      </c>
+      <c r="G43" s="5">
+        <f t="shared" si="18"/>
+        <v>4.7939597399576996</v>
+      </c>
+      <c r="H43" s="5"/>
+      <c r="I43" s="5">
+        <f t="shared" si="12"/>
+        <v>18134.622952599999</v>
+      </c>
+      <c r="J43" s="5">
+        <f t="shared" si="13"/>
+        <v>18309.113074557259</v>
+      </c>
+      <c r="K43" s="5">
+        <f t="shared" si="19"/>
+        <v>174.49012195726027</v>
+      </c>
+      <c r="M43" s="3">
+        <f t="shared" si="15"/>
+        <v>18138.021095697339</v>
+      </c>
+      <c r="N43" s="3">
+        <f t="shared" si="16"/>
+        <v>3.3981430973399256</v>
+      </c>
+    </row>
+    <row r="44" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B44" s="5">
+        <f t="shared" si="14"/>
+        <v>4064.1876352000004</v>
+      </c>
+      <c r="C44" s="5">
+        <f t="shared" si="9"/>
+        <v>4076.6612594394715</v>
+      </c>
+      <c r="D44" s="3">
+        <f t="shared" si="17"/>
+        <v>12.473624239471064</v>
+      </c>
+      <c r="E44" s="5">
+        <f t="shared" si="10"/>
+        <v>2712.4823726000004</v>
+      </c>
+      <c r="F44" s="5">
+        <f t="shared" si="11"/>
+        <v>2711.7534129652836</v>
+      </c>
+      <c r="G44" s="5">
+        <f t="shared" si="18"/>
+        <v>0.7289596347168299</v>
+      </c>
+      <c r="H44" s="5"/>
+      <c r="I44" s="5">
+        <f t="shared" si="12"/>
+        <v>20398.048878900001</v>
+      </c>
+      <c r="J44" s="5">
+        <f t="shared" si="13"/>
+        <v>20574.941852056458</v>
+      </c>
+      <c r="K44" s="5">
+        <f t="shared" si="19"/>
+        <v>176.89297315645672</v>
+      </c>
+      <c r="M44" s="3">
+        <f t="shared" si="15"/>
+        <v>20383.916470943092</v>
+      </c>
+      <c r="N44" s="3">
+        <f t="shared" si="16"/>
+        <v>14.132407956909447</v>
+      </c>
+    </row>
+    <row r="45" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B45" s="5">
+        <f t="shared" si="14"/>
+        <v>4064.1876352000004</v>
+      </c>
+      <c r="C45" s="5">
+        <f t="shared" si="9"/>
+        <v>4093.7900882606455</v>
+      </c>
+      <c r="D45" s="3">
+        <f t="shared" si="17"/>
+        <v>29.602453060645075</v>
+      </c>
+      <c r="E45" s="5">
+        <f t="shared" si="10"/>
+        <v>2712.4823726000004</v>
+      </c>
+      <c r="F45" s="5">
+        <f t="shared" si="11"/>
+        <v>2722.7992517146326</v>
+      </c>
+      <c r="G45" s="5">
+        <f t="shared" si="18"/>
+        <v>10.316879114632229</v>
+      </c>
+      <c r="H45" s="5"/>
+      <c r="I45" s="5">
+        <f t="shared" si="12"/>
+        <v>21804.185225900001</v>
+      </c>
+      <c r="J45" s="5">
+        <f t="shared" si="13"/>
+        <v>22019.597784019032</v>
+      </c>
+      <c r="K45" s="5">
+        <f t="shared" si="19"/>
+        <v>215.41255811903102</v>
+      </c>
+      <c r="M45" s="3">
+        <f t="shared" si="15"/>
+        <v>21815.863186703806</v>
+      </c>
+      <c r="N45" s="3">
+        <f t="shared" si="16"/>
+        <v>11.677960803805036</v>
+      </c>
+    </row>
+    <row r="46" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B46" s="5">
+        <f t="shared" si="14"/>
+        <v>4064.1876352000004</v>
+      </c>
+      <c r="C46" s="5">
+        <f t="shared" si="9"/>
+        <v>4088.0804786535878</v>
+      </c>
+      <c r="D46" s="3">
+        <f t="shared" si="17"/>
+        <v>23.892843453587375</v>
+      </c>
+      <c r="E46" s="5">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="F46" s="5">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="G46" s="5">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="H46" s="5"/>
+      <c r="I46" s="5">
+        <f t="shared" si="12"/>
+        <v>21804.185225900001</v>
+      </c>
+      <c r="J46" s="5">
+        <f t="shared" si="13"/>
+        <v>22019.597784019032</v>
+      </c>
+      <c r="K46" s="5">
+        <f t="shared" si="19"/>
+        <v>215.41255811903102</v>
+      </c>
+      <c r="M46" s="3">
+        <f t="shared" si="15"/>
+        <v>21815.863186703806</v>
+      </c>
+      <c r="N46" s="3">
+        <f t="shared" si="16"/>
+        <v>11.677960803805036</v>
+      </c>
+    </row>
+    <row r="47" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B47" s="5">
+        <f t="shared" si="14"/>
+        <v>4064.1876352000004</v>
+      </c>
+      <c r="C47" s="5">
+        <f t="shared" si="9"/>
+        <v>4096.6448930641745</v>
+      </c>
+      <c r="D47" s="3">
+        <f t="shared" si="17"/>
+        <v>32.457257864174153</v>
+      </c>
+      <c r="E47" s="5">
+        <f t="shared" si="10"/>
+        <v>2712.4823726000004</v>
+      </c>
+      <c r="F47" s="5">
+        <f t="shared" si="11"/>
+        <v>2722.7992517146326</v>
+      </c>
+      <c r="G47" s="5">
+        <f t="shared" si="18"/>
+        <v>10.316879114632229</v>
+      </c>
+      <c r="H47" s="5"/>
+      <c r="I47" s="5">
+        <f t="shared" si="12"/>
+        <v>16401.9000992</v>
+      </c>
+      <c r="J47" s="5">
+        <f t="shared" si="13"/>
+        <v>16545.112147108222</v>
+      </c>
+      <c r="K47" s="5">
+        <f t="shared" si="19"/>
+        <v>143.2120479082223</v>
+      </c>
+      <c r="M47" s="3">
+        <f t="shared" si="15"/>
+        <v>16389.538790136881</v>
+      </c>
+      <c r="N47" s="3">
+        <f t="shared" si="16"/>
+        <v>12.361309063118824</v>
+      </c>
+    </row>
+    <row r="48" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B48" s="5">
+        <f t="shared" si="14"/>
+        <v>4064.1876352000004</v>
+      </c>
+      <c r="C48" s="5">
+        <f t="shared" si="9"/>
         <v>4068.0968450288842</v>
       </c>
-      <c r="D37" s="3">
-        <f t="shared" ref="D37:D54" si="18">ABS(C37-B37)</f>
+      <c r="D48" s="3">
+        <f t="shared" si="17"/>
         <v>3.9092098288838315</v>
       </c>
-      <c r="E37" s="5">
+      <c r="E48" s="5">
+        <f t="shared" si="10"/>
+        <v>2712.4823726000004</v>
+      </c>
+      <c r="F48" s="5">
         <f t="shared" si="11"/>
+        <v>2722.7992517146326</v>
+      </c>
+      <c r="G48" s="5">
+        <f t="shared" si="18"/>
+        <v>10.316879114632229</v>
+      </c>
+      <c r="H48" s="5"/>
+      <c r="I48" s="5">
+        <f t="shared" si="12"/>
+        <v>12473.790175</v>
+      </c>
+      <c r="J48" s="5">
+        <f t="shared" si="13"/>
+        <v>12591.316964894861</v>
+      </c>
+      <c r="K48" s="5">
+        <f t="shared" si="19"/>
+        <v>117.52678989486049</v>
+      </c>
+      <c r="M48" s="3">
+        <f t="shared" si="15"/>
+        <v>12470.526725949665</v>
+      </c>
+      <c r="N48" s="3">
+        <f t="shared" si="16"/>
+        <v>3.2634490503351117</v>
+      </c>
+    </row>
+    <row r="49" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B49" s="5">
+        <f t="shared" si="14"/>
+        <v>4064.1876352000004</v>
+      </c>
+      <c r="C49" s="5">
+        <f t="shared" si="9"/>
+        <v>4085.2256738500591</v>
+      </c>
+      <c r="D49" s="3">
+        <f t="shared" si="17"/>
+        <v>21.038038650058752</v>
+      </c>
+      <c r="E49" s="5">
+        <f t="shared" si="10"/>
         <v>2712.4823726000004</v>
       </c>
-      <c r="F37" s="5">
+      <c r="F49" s="5">
+        <f t="shared" si="11"/>
+        <v>2722.7992517146326</v>
+      </c>
+      <c r="G49" s="5">
+        <f t="shared" si="18"/>
+        <v>10.316879114632229</v>
+      </c>
+      <c r="H49" s="5"/>
+      <c r="I49" s="5">
         <f t="shared" si="12"/>
-        <v>2733.8450904639822</v>
-      </c>
-      <c r="G37" s="5">
-        <f t="shared" ref="G37:G54" si="19">ABS(F37-E37)</f>
-        <v>21.362717863981743</v>
-      </c>
-      <c r="H37" s="5">
+        <v>8445.8899294000003</v>
+      </c>
+      <c r="J49" s="5">
         <f t="shared" si="13"/>
+        <v>8561.4872599466271</v>
+      </c>
+      <c r="K49" s="5">
+        <f t="shared" si="19"/>
+        <v>115.59733054662684</v>
+      </c>
+      <c r="M49" s="3">
+        <f t="shared" si="15"/>
+        <v>8476.1490451434602</v>
+      </c>
+      <c r="N49" s="3">
+        <f t="shared" si="16"/>
+        <v>30.259115743459915</v>
+      </c>
+    </row>
+    <row r="50" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B50" s="5">
+        <f t="shared" si="14"/>
+        <v>4064.1876352000004</v>
+      </c>
+      <c r="C50" s="5">
+        <f t="shared" si="9"/>
+        <v>4088.0804786535878</v>
+      </c>
+      <c r="D50" s="3">
+        <f t="shared" si="17"/>
+        <v>23.892843453587375</v>
+      </c>
+      <c r="E50" s="5">
+        <f t="shared" si="10"/>
+        <v>2712.4823726000004</v>
+      </c>
+      <c r="F50" s="5">
+        <f t="shared" si="11"/>
+        <v>2717.2763323399581</v>
+      </c>
+      <c r="G50" s="5">
+        <f t="shared" si="18"/>
+        <v>4.7939597399576996</v>
+      </c>
+      <c r="H50" s="5"/>
+      <c r="I50" s="5">
+        <f t="shared" si="12"/>
+        <v>4930.5490619000002</v>
+      </c>
+      <c r="J50" s="5">
+        <f t="shared" si="13"/>
+        <v>4987.8646914076262</v>
+      </c>
+      <c r="K50" s="5">
+        <f t="shared" si="19"/>
+        <v>57.315629507625999</v>
+      </c>
+      <c r="M50" s="3">
+        <f t="shared" si="15"/>
+        <v>4933.9650640511654</v>
+      </c>
+      <c r="N50" s="3">
+        <f t="shared" si="16"/>
+        <v>3.4160021511652303</v>
+      </c>
+    </row>
+    <row r="51" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B51" s="5">
+        <f t="shared" si="14"/>
+        <v>4064.1876352000004</v>
+      </c>
+      <c r="C51" s="5">
+        <f t="shared" si="9"/>
+        <v>4085.2256738500591</v>
+      </c>
+      <c r="D51" s="3">
+        <f t="shared" si="17"/>
+        <v>21.038038650058752</v>
+      </c>
+      <c r="E51" s="5">
+        <f t="shared" si="10"/>
+        <v>2712.4823726000004</v>
+      </c>
+      <c r="F51" s="5">
+        <f t="shared" si="11"/>
+        <v>2722.7992517146326</v>
+      </c>
+      <c r="G51" s="5">
+        <f t="shared" si="18"/>
+        <v>10.316879114632229</v>
+      </c>
+      <c r="H51" s="5"/>
+      <c r="I51" s="5">
+        <f t="shared" si="12"/>
+        <v>2290.6414685</v>
+      </c>
+      <c r="J51" s="5">
+        <f>U27*453.59237</f>
+        <v>2326.6563956870941</v>
+      </c>
+      <c r="K51" s="5">
+        <f t="shared" si="19"/>
+        <v>36.014927187094145</v>
+      </c>
+      <c r="M51" s="3">
+        <f t="shared" si="15"/>
+        <v>2296.1684823866908</v>
+      </c>
+      <c r="N51" s="3">
+        <f t="shared" si="16"/>
+        <v>5.5270138866908383</v>
+      </c>
+    </row>
+    <row r="52" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B52" s="5">
+        <f t="shared" si="14"/>
+        <v>4064.1876352000004</v>
+      </c>
+      <c r="C52" s="5">
+        <f t="shared" si="9"/>
+        <v>4068.0968450288842</v>
+      </c>
+      <c r="D52" s="3">
+        <f t="shared" si="17"/>
+        <v>3.9092098288838315</v>
+      </c>
+      <c r="E52" s="5">
+        <f t="shared" si="10"/>
+        <v>2712.4823726000004</v>
+      </c>
+      <c r="F52" s="5">
+        <f t="shared" si="11"/>
+        <v>2708.9919532779459</v>
+      </c>
+      <c r="G52" s="5">
+        <f t="shared" si="18"/>
+        <v>3.4904193220545494</v>
+      </c>
+      <c r="H52" s="5"/>
+      <c r="I52" s="5">
+        <f t="shared" si="12"/>
         <v>802.85849489999998</v>
       </c>
-      <c r="I37" s="5">
+      <c r="J52" s="5">
+        <f>U28*453.59237</f>
+        <v>836.3797500835957</v>
+      </c>
+      <c r="K52" s="5">
+        <f t="shared" si="19"/>
+        <v>33.521255183595713</v>
+      </c>
+      <c r="M52" s="3">
+        <f t="shared" si="15"/>
+        <v>819.0023966545848</v>
+      </c>
+      <c r="N52" s="3">
+        <f t="shared" si="16"/>
+        <v>16.143901754584817</v>
+      </c>
+    </row>
+    <row r="53" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B53" s="5">
         <f t="shared" si="14"/>
-        <v>821.17284553662125</v>
-      </c>
-      <c r="J37" s="5">
-        <f t="shared" ref="J37:J54" si="20">ABS(I37-H37)</f>
-        <v>18.31435063662127</v>
-      </c>
-      <c r="L37" s="3">
-        <f t="shared" si="16"/>
-        <v>803.92927333078785</v>
-      </c>
-      <c r="M37" s="3">
+        <v>4064.1876352000004</v>
+      </c>
+      <c r="C53" s="5">
+        <f t="shared" si="9"/>
+        <v>4085.2256738500591</v>
+      </c>
+      <c r="D53" s="3">
         <f t="shared" si="17"/>
-        <v>1.0707784307878683</v>
-      </c>
-    </row>
-    <row r="38" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B38" s="5">
+        <v>21.038038650058752</v>
+      </c>
+      <c r="E53" s="5">
+        <f t="shared" si="10"/>
+        <v>2712.4823726000004</v>
+      </c>
+      <c r="F53" s="5">
+        <f t="shared" si="11"/>
+        <v>2714.5148726526204</v>
+      </c>
+      <c r="G53" s="5">
+        <f t="shared" si="18"/>
+        <v>2.0325000526199801</v>
+      </c>
+      <c r="H53" s="5"/>
+      <c r="I53" s="5">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J53" s="5">
+        <f>U29*453.59237</f>
+        <v>15.206904546974464</v>
+      </c>
+      <c r="K53" s="5">
+        <f t="shared" si="19"/>
+        <v>15.206904546974464</v>
+      </c>
+      <c r="M53" s="3">
         <f t="shared" si="15"/>
-        <v>4064.1876352000004</v>
-      </c>
-      <c r="C38" s="5">
-        <f t="shared" si="10"/>
-        <v>4082.3708690465301</v>
-      </c>
-      <c r="D38" s="3">
-        <f t="shared" si="18"/>
-        <v>18.183233846529674</v>
-      </c>
-      <c r="E38" s="5">
-        <f t="shared" si="11"/>
-        <v>2712.4823726000004</v>
-      </c>
-      <c r="F38" s="5">
-        <f t="shared" si="12"/>
-        <v>2744.8909292133321</v>
-      </c>
-      <c r="G38" s="5">
-        <f t="shared" si="19"/>
-        <v>32.408556613331712</v>
-      </c>
-      <c r="H38" s="5">
-        <f t="shared" si="13"/>
-        <v>2345.0725529000001</v>
-      </c>
-      <c r="I38" s="5">
-        <f t="shared" si="14"/>
-        <v>2357.0702047810428</v>
-      </c>
-      <c r="J38" s="5">
-        <f t="shared" si="20"/>
-        <v>11.997651881042657</v>
-      </c>
-      <c r="L38" s="3">
-        <f t="shared" si="16"/>
-        <v>2326.3147290342849</v>
-      </c>
-      <c r="M38" s="3">
-        <f t="shared" si="17"/>
-        <v>18.757823865715181</v>
-      </c>
-    </row>
-    <row r="39" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B39" s="5">
-        <f t="shared" si="15"/>
-        <v>4064.1876352000004</v>
-      </c>
-      <c r="C39" s="5">
-        <f t="shared" si="10"/>
-        <v>4090.9352834571168</v>
-      </c>
-      <c r="D39" s="3">
-        <f t="shared" si="18"/>
-        <v>26.747648257116452</v>
-      </c>
-      <c r="E39" s="5">
-        <f t="shared" si="11"/>
-        <v>2712.4823726000004</v>
-      </c>
-      <c r="F39" s="5">
-        <f t="shared" si="12"/>
-        <v>2714.5148726526204</v>
-      </c>
-      <c r="G39" s="5">
-        <f t="shared" si="19"/>
-        <v>2.0325000526199801</v>
-      </c>
-      <c r="H39" s="5">
-        <f t="shared" si="13"/>
-        <v>5102.9141625000002</v>
-      </c>
-      <c r="I39" s="5">
-        <f t="shared" si="14"/>
-        <v>5155.1406414243447</v>
-      </c>
-      <c r="J39" s="5">
-        <f t="shared" si="20"/>
-        <v>52.226478924344519</v>
-      </c>
-      <c r="L39" s="3">
-        <f t="shared" si="16"/>
-        <v>5099.7694206129327</v>
-      </c>
-      <c r="M39" s="3">
-        <f t="shared" si="17"/>
-        <v>3.1447418870675392</v>
-      </c>
-    </row>
-    <row r="40" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B40" s="5">
-        <f t="shared" si="15"/>
-        <v>4064.1876352000004</v>
-      </c>
-      <c r="C40" s="5">
-        <f t="shared" si="10"/>
-        <v>4082.3708690465301</v>
-      </c>
-      <c r="D40" s="3">
-        <f t="shared" si="18"/>
-        <v>18.183233846529674</v>
-      </c>
-      <c r="E40" s="5">
-        <f t="shared" si="11"/>
-        <v>2712.4823726000004</v>
-      </c>
-      <c r="F40" s="5">
-        <f t="shared" si="12"/>
-        <v>2722.7992517146326</v>
-      </c>
-      <c r="G40" s="5">
-        <f t="shared" si="19"/>
-        <v>10.316879114632229</v>
-      </c>
-      <c r="H40" s="5">
-        <f t="shared" si="13"/>
-        <v>8600.1113352000011</v>
-      </c>
-      <c r="I40" s="5">
-        <f t="shared" si="14"/>
-        <v>8683.1424963224217</v>
-      </c>
-      <c r="J40" s="5">
-        <f t="shared" si="20"/>
-        <v>83.031161122420599</v>
-      </c>
-      <c r="L40" s="3">
-        <f t="shared" si="16"/>
-        <v>8596.7340317338367</v>
-      </c>
-      <c r="M40" s="3">
-        <f t="shared" si="17"/>
-        <v>3.3773034661644488</v>
-      </c>
-    </row>
-    <row r="41" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B41" s="5">
-        <f t="shared" si="15"/>
-        <v>4064.1876352000004</v>
-      </c>
-      <c r="C41" s="5">
-        <f t="shared" si="10"/>
-        <v>4079.5160642430005</v>
-      </c>
-      <c r="D41" s="3">
-        <f t="shared" si="18"/>
-        <v>15.328429043000142</v>
-      </c>
-      <c r="E41" s="5">
-        <f t="shared" si="11"/>
-        <v>2712.4823726000004</v>
-      </c>
-      <c r="F41" s="5">
-        <f t="shared" si="12"/>
-        <v>2720.0377920272958</v>
-      </c>
-      <c r="G41" s="5">
-        <f t="shared" si="19"/>
-        <v>7.5554194272954192</v>
-      </c>
-      <c r="H41" s="5">
-        <f t="shared" si="13"/>
-        <v>12451.1105565</v>
-      </c>
-      <c r="I41" s="5">
-        <f t="shared" si="14"/>
-        <v>12560.90315580091</v>
-      </c>
-      <c r="J41" s="5">
-        <f t="shared" si="20"/>
-        <v>109.7925993009103</v>
-      </c>
-      <c r="L41" s="3">
-        <f t="shared" si="16"/>
-        <v>12440.380479302072</v>
-      </c>
-      <c r="M41" s="3">
-        <f t="shared" si="17"/>
-        <v>10.73007719792804</v>
-      </c>
-    </row>
-    <row r="42" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B42" s="5">
-        <f t="shared" si="15"/>
-        <v>4064.1876352000004</v>
-      </c>
-      <c r="C42" s="5">
-        <f t="shared" si="10"/>
-        <v>4070.9516498324128</v>
-      </c>
-      <c r="D42" s="3">
-        <f t="shared" si="18"/>
-        <v>6.7640146324124544</v>
-      </c>
-      <c r="E42" s="5">
-        <f t="shared" si="11"/>
-        <v>2712.4823726000004</v>
-      </c>
-      <c r="F42" s="5">
-        <f t="shared" si="12"/>
-        <v>2733.8450904639822</v>
-      </c>
-      <c r="G42" s="5">
-        <f t="shared" si="19"/>
-        <v>21.362717863981743</v>
-      </c>
-      <c r="H42" s="5">
-        <f t="shared" si="13"/>
-        <v>15794.086323400001</v>
-      </c>
-      <c r="I42" s="5">
-        <f t="shared" si="14"/>
-        <v>15936.83596522924</v>
-      </c>
-      <c r="J42" s="5">
-        <f t="shared" si="20"/>
-        <v>142.74964182923941</v>
-      </c>
-      <c r="L42" s="3">
-        <f t="shared" si="16"/>
-        <v>15786.613857185004</v>
-      </c>
-      <c r="M42" s="3">
-        <f t="shared" si="17"/>
-        <v>7.4724662149965297</v>
-      </c>
-    </row>
-    <row r="43" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B43" s="5">
-        <f t="shared" si="15"/>
-        <v>4064.1876352000004</v>
-      </c>
-      <c r="C43" s="5">
-        <f t="shared" si="10"/>
-        <v>4082.3708690465301</v>
-      </c>
-      <c r="D43" s="3">
-        <f t="shared" si="18"/>
-        <v>18.183233846529674</v>
-      </c>
-      <c r="E43" s="5">
-        <f t="shared" si="11"/>
-        <v>2712.4823726000004</v>
-      </c>
-      <c r="F43" s="5">
-        <f t="shared" si="12"/>
-        <v>2717.2763323399581</v>
-      </c>
-      <c r="G43" s="5">
-        <f t="shared" si="19"/>
-        <v>4.7939597399576996</v>
-      </c>
-      <c r="H43" s="5">
-        <f t="shared" si="13"/>
-        <v>18134.622952599999</v>
-      </c>
-      <c r="I43" s="5">
-        <f t="shared" si="14"/>
-        <v>18309.113074557259</v>
-      </c>
-      <c r="J43" s="5">
-        <f t="shared" si="20"/>
-        <v>174.49012195726027</v>
-      </c>
-      <c r="L43" s="3">
-        <f t="shared" si="16"/>
-        <v>18138.021095697339</v>
-      </c>
-      <c r="M43" s="3">
-        <f t="shared" si="17"/>
-        <v>3.3981430973399256</v>
-      </c>
-    </row>
-    <row r="44" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B44" s="5">
-        <f t="shared" si="15"/>
-        <v>4064.1876352000004</v>
-      </c>
-      <c r="C44" s="5">
-        <f t="shared" si="10"/>
-        <v>4076.6612594394715</v>
-      </c>
-      <c r="D44" s="3">
-        <f t="shared" si="18"/>
-        <v>12.473624239471064</v>
-      </c>
-      <c r="E44" s="5">
-        <f t="shared" si="11"/>
-        <v>2712.4823726000004</v>
-      </c>
-      <c r="F44" s="5">
-        <f t="shared" si="12"/>
-        <v>2711.7534129652836</v>
-      </c>
-      <c r="G44" s="5">
-        <f t="shared" si="19"/>
-        <v>0.7289596347168299</v>
-      </c>
-      <c r="H44" s="5">
-        <f t="shared" si="13"/>
-        <v>20398.048878900001</v>
-      </c>
-      <c r="I44" s="5">
-        <f t="shared" si="14"/>
-        <v>20574.941852056458</v>
-      </c>
-      <c r="J44" s="5">
-        <f t="shared" si="20"/>
-        <v>176.89297315645672</v>
-      </c>
-      <c r="L44" s="3">
-        <f t="shared" si="16"/>
-        <v>20383.916470943092</v>
-      </c>
-      <c r="M44" s="3">
-        <f t="shared" si="17"/>
-        <v>14.132407956909447</v>
-      </c>
-    </row>
-    <row r="45" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B45" s="5">
-        <f t="shared" si="15"/>
-        <v>4064.1876352000004</v>
-      </c>
-      <c r="C45" s="5">
-        <f t="shared" si="10"/>
-        <v>4093.7900882606455</v>
-      </c>
-      <c r="D45" s="3">
-        <f t="shared" si="18"/>
-        <v>29.602453060645075</v>
-      </c>
-      <c r="E45" s="5">
-        <f t="shared" si="11"/>
-        <v>2712.4823726000004</v>
-      </c>
-      <c r="F45" s="5">
-        <f t="shared" si="12"/>
-        <v>2722.7992517146326</v>
-      </c>
-      <c r="G45" s="5">
-        <f t="shared" si="19"/>
-        <v>10.316879114632229</v>
-      </c>
-      <c r="H45" s="5">
-        <f t="shared" si="13"/>
-        <v>21804.185225900001</v>
-      </c>
-      <c r="I45" s="5">
-        <f t="shared" si="14"/>
-        <v>22019.597784019032</v>
-      </c>
-      <c r="J45" s="5">
-        <f t="shared" si="20"/>
-        <v>215.41255811903102</v>
-      </c>
-      <c r="L45" s="3">
-        <f t="shared" si="16"/>
-        <v>21815.863186703806</v>
-      </c>
-      <c r="M45" s="3">
-        <f t="shared" si="17"/>
-        <v>11.677960803805036</v>
-      </c>
-    </row>
-    <row r="46" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B46" s="5">
-        <f t="shared" si="15"/>
-        <v>4064.1876352000004</v>
-      </c>
-      <c r="C46" s="5">
-        <f t="shared" si="10"/>
-        <v>4088.0804786535878</v>
-      </c>
-      <c r="D46" s="3">
-        <f t="shared" si="18"/>
-        <v>23.892843453587375</v>
-      </c>
-      <c r="E46" s="5">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="F46" s="5">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="G46" s="5">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-      <c r="H46" s="5">
-        <f t="shared" si="13"/>
-        <v>21804.185225900001</v>
-      </c>
-      <c r="I46" s="5">
-        <f t="shared" si="14"/>
-        <v>22019.597784019032</v>
-      </c>
-      <c r="J46" s="5">
-        <f t="shared" si="20"/>
-        <v>215.41255811903102</v>
-      </c>
-      <c r="L46" s="3">
-        <f t="shared" si="16"/>
-        <v>21815.863186703806</v>
-      </c>
-      <c r="M46" s="3">
-        <f t="shared" si="17"/>
-        <v>11.677960803805036</v>
-      </c>
-    </row>
-    <row r="47" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B47" s="5">
-        <f t="shared" si="15"/>
-        <v>4064.1876352000004</v>
-      </c>
-      <c r="C47" s="5">
-        <f t="shared" si="10"/>
-        <v>4096.6448930641745</v>
-      </c>
-      <c r="D47" s="3">
-        <f t="shared" si="18"/>
-        <v>32.457257864174153</v>
-      </c>
-      <c r="E47" s="5">
-        <f t="shared" si="11"/>
-        <v>2712.4823726000004</v>
-      </c>
-      <c r="F47" s="5">
-        <f t="shared" si="12"/>
-        <v>2722.7992517146326</v>
-      </c>
-      <c r="G47" s="5">
-        <f t="shared" si="19"/>
-        <v>10.316879114632229</v>
-      </c>
-      <c r="H47" s="5">
-        <f t="shared" si="13"/>
-        <v>16401.9000992</v>
-      </c>
-      <c r="I47" s="5">
-        <f t="shared" si="14"/>
-        <v>16545.112147108222</v>
-      </c>
-      <c r="J47" s="5">
-        <f t="shared" si="20"/>
-        <v>143.2120479082223</v>
-      </c>
-      <c r="L47" s="3">
-        <f t="shared" si="16"/>
-        <v>16389.538790136881</v>
-      </c>
-      <c r="M47" s="3">
-        <f t="shared" si="17"/>
-        <v>12.361309063118824</v>
-      </c>
-    </row>
-    <row r="48" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B48" s="5">
-        <f t="shared" si="15"/>
-        <v>4064.1876352000004</v>
-      </c>
-      <c r="C48" s="5">
-        <f t="shared" si="10"/>
-        <v>4068.0968450288842</v>
-      </c>
-      <c r="D48" s="3">
-        <f t="shared" si="18"/>
-        <v>3.9092098288838315</v>
-      </c>
-      <c r="E48" s="5">
-        <f t="shared" si="11"/>
-        <v>2712.4823726000004</v>
-      </c>
-      <c r="F48" s="5">
-        <f t="shared" si="12"/>
-        <v>2722.7992517146326</v>
-      </c>
-      <c r="G48" s="5">
-        <f t="shared" si="19"/>
-        <v>10.316879114632229</v>
-      </c>
-      <c r="H48" s="5">
-        <f t="shared" si="13"/>
-        <v>12473.790175</v>
-      </c>
-      <c r="I48" s="5">
-        <f t="shared" si="14"/>
-        <v>12591.316964894861</v>
-      </c>
-      <c r="J48" s="5">
-        <f t="shared" si="20"/>
-        <v>117.52678989486049</v>
-      </c>
-      <c r="L48" s="3">
-        <f t="shared" si="16"/>
-        <v>12470.526725949665</v>
-      </c>
-      <c r="M48" s="3">
-        <f t="shared" si="17"/>
-        <v>3.2634490503351117</v>
-      </c>
-    </row>
-    <row r="49" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B49" s="5">
-        <f t="shared" si="15"/>
-        <v>4064.1876352000004</v>
-      </c>
-      <c r="C49" s="5">
-        <f t="shared" si="10"/>
-        <v>4085.2256738500591</v>
-      </c>
-      <c r="D49" s="3">
-        <f t="shared" si="18"/>
-        <v>21.038038650058752</v>
-      </c>
-      <c r="E49" s="5">
-        <f t="shared" si="11"/>
-        <v>2712.4823726000004</v>
-      </c>
-      <c r="F49" s="5">
-        <f t="shared" si="12"/>
-        <v>2722.7992517146326</v>
-      </c>
-      <c r="G49" s="5">
-        <f t="shared" si="19"/>
-        <v>10.316879114632229</v>
-      </c>
-      <c r="H49" s="5">
-        <f t="shared" si="13"/>
-        <v>8445.8899294000003</v>
-      </c>
-      <c r="I49" s="5">
-        <f t="shared" si="14"/>
-        <v>8561.4872599466271</v>
-      </c>
-      <c r="J49" s="5">
-        <f t="shared" si="20"/>
-        <v>115.59733054662684</v>
-      </c>
-      <c r="L49" s="3">
-        <f t="shared" si="16"/>
-        <v>8476.1490451434602</v>
-      </c>
-      <c r="M49" s="3">
-        <f t="shared" si="17"/>
-        <v>30.259115743459915</v>
-      </c>
-    </row>
-    <row r="50" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B50" s="5">
-        <f t="shared" si="15"/>
-        <v>4064.1876352000004</v>
-      </c>
-      <c r="C50" s="5">
-        <f t="shared" si="10"/>
-        <v>4088.0804786535878</v>
-      </c>
-      <c r="D50" s="3">
-        <f t="shared" si="18"/>
-        <v>23.892843453587375</v>
-      </c>
-      <c r="E50" s="5">
-        <f t="shared" si="11"/>
-        <v>2712.4823726000004</v>
-      </c>
-      <c r="F50" s="5">
-        <f t="shared" si="12"/>
-        <v>2717.2763323399581</v>
-      </c>
-      <c r="G50" s="5">
-        <f t="shared" si="19"/>
-        <v>4.7939597399576996</v>
-      </c>
-      <c r="H50" s="5">
-        <f t="shared" si="13"/>
-        <v>4930.5490619000002</v>
-      </c>
-      <c r="I50" s="5">
-        <f t="shared" si="14"/>
-        <v>4987.8646914076262</v>
-      </c>
-      <c r="J50" s="5">
-        <f t="shared" si="20"/>
-        <v>57.315629507625999</v>
-      </c>
-      <c r="L50" s="3">
-        <f t="shared" si="16"/>
-        <v>4933.9650640511654</v>
-      </c>
-      <c r="M50" s="3">
-        <f t="shared" si="17"/>
-        <v>3.4160021511652303</v>
-      </c>
-    </row>
-    <row r="51" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B51" s="5">
-        <f t="shared" si="15"/>
-        <v>4064.1876352000004</v>
-      </c>
-      <c r="C51" s="5">
-        <f t="shared" si="10"/>
-        <v>4085.2256738500591</v>
-      </c>
-      <c r="D51" s="3">
-        <f t="shared" si="18"/>
-        <v>21.038038650058752</v>
-      </c>
-      <c r="E51" s="5">
-        <f t="shared" si="11"/>
-        <v>2712.4823726000004</v>
-      </c>
-      <c r="F51" s="5">
-        <f t="shared" si="12"/>
-        <v>2722.7992517146326</v>
-      </c>
-      <c r="G51" s="5">
-        <f t="shared" si="19"/>
-        <v>10.316879114632229</v>
-      </c>
-      <c r="H51" s="5">
-        <f t="shared" si="13"/>
-        <v>2290.6414685</v>
-      </c>
-      <c r="I51" s="5">
-        <f>T27*453.59237</f>
-        <v>2326.6563956870941</v>
-      </c>
-      <c r="J51" s="5">
-        <f t="shared" si="20"/>
-        <v>36.014927187094145</v>
-      </c>
-      <c r="L51" s="3">
-        <f t="shared" si="16"/>
-        <v>2296.1684823866908</v>
-      </c>
-      <c r="M51" s="3">
-        <f t="shared" si="17"/>
-        <v>5.5270138866908383</v>
-      </c>
-    </row>
-    <row r="52" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B52" s="5">
-        <f t="shared" si="15"/>
-        <v>4064.1876352000004</v>
-      </c>
-      <c r="C52" s="5">
-        <f t="shared" si="10"/>
-        <v>4068.0968450288842</v>
-      </c>
-      <c r="D52" s="3">
-        <f t="shared" si="18"/>
-        <v>3.9092098288838315</v>
-      </c>
-      <c r="E52" s="5">
-        <f t="shared" si="11"/>
-        <v>2712.4823726000004</v>
-      </c>
-      <c r="F52" s="5">
-        <f t="shared" si="12"/>
-        <v>2708.9919532779459</v>
-      </c>
-      <c r="G52" s="5">
-        <f t="shared" si="19"/>
-        <v>3.4904193220545494</v>
-      </c>
-      <c r="H52" s="5">
-        <f t="shared" si="13"/>
-        <v>802.85849489999998</v>
-      </c>
-      <c r="I52" s="5">
-        <f>T28*453.59237</f>
-        <v>836.3797500835957</v>
-      </c>
-      <c r="J52" s="5">
-        <f t="shared" si="20"/>
-        <v>33.521255183595713</v>
-      </c>
-      <c r="L52" s="3">
-        <f t="shared" si="16"/>
-        <v>819.0023966545848</v>
-      </c>
-      <c r="M52" s="3">
-        <f t="shared" si="17"/>
-        <v>16.143901754584817</v>
-      </c>
-    </row>
-    <row r="53" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B53" s="5">
-        <f t="shared" si="15"/>
-        <v>4064.1876352000004</v>
-      </c>
-      <c r="C53" s="5">
-        <f t="shared" si="10"/>
-        <v>4085.2256738500591</v>
-      </c>
-      <c r="D53" s="3">
-        <f t="shared" si="18"/>
-        <v>21.038038650058752</v>
-      </c>
-      <c r="E53" s="5">
-        <f t="shared" si="11"/>
-        <v>2712.4823726000004</v>
-      </c>
-      <c r="F53" s="5">
-        <f t="shared" si="12"/>
-        <v>2714.5148726526204</v>
-      </c>
-      <c r="G53" s="5">
-        <f t="shared" si="19"/>
-        <v>2.0325000526199801</v>
-      </c>
-      <c r="H53" s="5">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="I53" s="5">
-        <f>T29*453.59237</f>
-        <v>15.206904546974464</v>
-      </c>
-      <c r="J53" s="5">
-        <f t="shared" si="20"/>
-        <v>15.206904546974464</v>
-      </c>
-      <c r="L53" s="3">
+        <v>5.053737169546892</v>
+      </c>
+      <c r="N53" s="3">
         <f t="shared" si="16"/>
         <v>5.053737169546892</v>
       </c>
-      <c r="M53" s="3">
+    </row>
+    <row r="54" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B54" s="5">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="C54" s="5">
+        <f t="shared" si="9"/>
+        <v>2.8548048035290443</v>
+      </c>
+      <c r="D54" s="3">
         <f t="shared" si="17"/>
+        <v>2.8548048035290443</v>
+      </c>
+      <c r="E54" s="5">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="F54" s="5">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="G54" s="5">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="H54" s="5"/>
+      <c r="I54" s="5">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J54" s="5">
+        <f>U30*453.59237</f>
+        <v>15.206904546974464</v>
+      </c>
+      <c r="K54" s="5">
+        <f t="shared" si="19"/>
+        <v>15.206904546974464</v>
+      </c>
+      <c r="M54" s="3">
+        <f t="shared" si="15"/>
         <v>5.053737169546892</v>
       </c>
-    </row>
-    <row r="54" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B54" s="5">
-        <f t="shared" si="15"/>
-        <v>0</v>
-      </c>
-      <c r="C54" s="5">
-        <f t="shared" si="10"/>
-        <v>2.8548048035290443</v>
-      </c>
-      <c r="D54" s="3">
-        <f t="shared" si="18"/>
-        <v>2.8548048035290443</v>
-      </c>
-      <c r="E54" s="5">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="F54" s="5">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="G54" s="5">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-      <c r="H54" s="5">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="I54" s="5">
-        <f>T30*453.59237</f>
-        <v>15.206904546974464</v>
-      </c>
-      <c r="J54" s="5">
-        <f t="shared" si="20"/>
-        <v>15.206904546974464</v>
-      </c>
-      <c r="L54" s="3">
+      <c r="N54" s="3">
         <f t="shared" si="16"/>
         <v>5.053737169546892</v>
       </c>
-      <c r="M54" s="3">
-        <f t="shared" si="17"/>
-        <v>5.053737169546892</v>
-      </c>
-    </row>
-    <row r="55" spans="2:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="55" spans="2:14" x14ac:dyDescent="0.25">
       <c r="C55" t="s">
         <v>40</v>
       </c>
@@ -3775,22 +3879,23 @@
         <f>AVERAGE(G39:G54)</f>
         <v>6.7932319075623298</v>
       </c>
-      <c r="I55" t="s">
+      <c r="H55" s="3"/>
+      <c r="J55" t="s">
         <v>40</v>
       </c>
-      <c r="J55" s="3">
-        <f>AVERAGE(J39:J54)</f>
+      <c r="K55" s="3">
+        <f>AVERAGE(K39:K54)</f>
         <v>106.47561761566678</v>
       </c>
-      <c r="L55" t="s">
+      <c r="M55" t="s">
         <v>40</v>
       </c>
-      <c r="M55" s="3">
-        <f>AVERAGE(M39:M54)</f>
+      <c r="N55" s="3">
+        <f>AVERAGE(N39:N54)</f>
         <v>9.1680829635290308</v>
       </c>
     </row>
-    <row r="56" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:14" x14ac:dyDescent="0.25">
       <c r="C56" t="s">
         <v>41</v>
       </c>
@@ -3805,22 +3910,23 @@
         <f>MIN(G40:G54)</f>
         <v>0</v>
       </c>
-      <c r="I56" t="s">
+      <c r="H56" s="3"/>
+      <c r="J56" t="s">
         <v>41</v>
       </c>
-      <c r="J56" s="3">
-        <f>MIN(J40:J54)</f>
+      <c r="K56" s="3">
+        <f>MIN(K40:K54)</f>
         <v>15.206904546974464</v>
       </c>
-      <c r="L56" t="s">
+      <c r="M56" t="s">
         <v>41</v>
       </c>
-      <c r="M56" s="3">
-        <f>MIN(M40:M54)</f>
+      <c r="N56" s="3">
+        <f>MIN(N40:N54)</f>
         <v>3.2634490503351117</v>
       </c>
     </row>
-    <row r="57" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:14" x14ac:dyDescent="0.25">
       <c r="C57" t="s">
         <v>42</v>
       </c>
@@ -3835,24 +3941,25 @@
         <f>MAX(G39:G54)</f>
         <v>21.362717863981743</v>
       </c>
-      <c r="I57" t="s">
+      <c r="H57" s="3"/>
+      <c r="J57" t="s">
         <v>42</v>
       </c>
-      <c r="J57" s="3">
-        <f>MAX(J39:J54)</f>
+      <c r="K57" s="3">
+        <f>MAX(K39:K54)</f>
         <v>215.41255811903102</v>
       </c>
-      <c r="L57" t="s">
+      <c r="M57" t="s">
         <v>42</v>
       </c>
-      <c r="M57" s="3">
-        <f>MAX(M39:M54)</f>
+      <c r="N57" s="3">
+        <f>MAX(N39:N54)</f>
         <v>30.259115743459915</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="G35:G54 J35:J54">
-    <cfRule type="colorScale" priority="2">
+  <conditionalFormatting sqref="D35:D54">
+    <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -3863,8 +3970,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D35:D54">
-    <cfRule type="colorScale" priority="1">
+  <conditionalFormatting sqref="G35:H54 K35:K54">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>